<commit_message>
Atualização automática: pagamentos (15/09/2026 08:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,8 +491,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -508,7 +516,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -516,12 +524,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -821,37 +847,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -901,58 +927,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -969,13 +995,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1010,13 +1036,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1051,13 +1077,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1092,13 +1118,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1133,13 +1159,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1177,13 +1203,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1218,13 +1244,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1259,13 +1285,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1297,13 +1323,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1338,13 +1364,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1379,13 +1405,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1417,13 +1443,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1455,13 +1481,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1496,13 +1522,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1537,13 +1563,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1578,13 +1604,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1619,13 +1645,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1660,13 +1686,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1701,13 +1727,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1736,13 +1762,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1777,13 +1803,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1821,13 +1847,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1865,13 +1891,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1909,13 +1935,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1950,13 +1976,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1991,13 +2017,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2032,13 +2058,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2073,13 +2099,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2171,13 +2197,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2209,13 +2235,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2248,19 +2274,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (15/09/2026 12:32)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,16 +491,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -516,7 +508,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -524,30 +516,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -847,37 +821,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -927,58 +901,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -995,13 +969,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1036,13 +1010,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1077,13 +1051,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1118,13 +1092,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1159,13 +1133,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1203,13 +1177,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1244,13 +1218,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1285,13 +1259,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1323,13 +1297,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1364,13 +1338,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1405,13 +1379,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1443,13 +1417,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1481,13 +1455,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1522,13 +1496,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1563,13 +1537,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1604,13 +1578,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1645,13 +1619,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1686,13 +1660,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1727,13 +1701,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1762,13 +1736,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1803,13 +1777,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1847,13 +1821,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1891,13 +1865,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1935,13 +1909,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1976,13 +1950,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2017,13 +1991,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2058,13 +2032,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2099,13 +2073,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2197,13 +2171,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2235,13 +2209,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2274,19 +2248,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (15/09/2026 14:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,8 +491,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -508,7 +516,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -516,12 +524,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -821,37 +847,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -901,58 +927,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -969,13 +995,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1010,13 +1036,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1051,13 +1077,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1092,13 +1118,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1133,13 +1159,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1177,13 +1203,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1218,13 +1244,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1259,13 +1285,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1297,13 +1323,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1338,13 +1364,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1379,13 +1405,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1417,13 +1443,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1455,13 +1481,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1496,13 +1522,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1537,13 +1563,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1578,13 +1604,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1619,13 +1645,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1660,13 +1686,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1701,13 +1727,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1736,13 +1762,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1777,13 +1803,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1821,13 +1847,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1865,13 +1891,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1909,13 +1935,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1950,13 +1976,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1991,13 +2017,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2032,13 +2058,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2073,13 +2099,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2171,13 +2197,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2209,13 +2235,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2248,19 +2274,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (16/09/2026 12:24)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,16 +491,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -516,7 +508,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -524,30 +516,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -847,37 +821,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -927,58 +901,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -995,13 +969,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1036,13 +1010,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1077,13 +1051,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1118,13 +1092,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1159,13 +1133,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1203,13 +1177,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1244,13 +1218,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1285,13 +1259,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1323,13 +1297,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1364,13 +1338,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1405,13 +1379,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1443,13 +1417,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1481,13 +1455,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1522,13 +1496,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1563,13 +1537,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1604,13 +1578,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1645,13 +1619,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1686,13 +1660,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1727,13 +1701,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1762,13 +1736,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1803,13 +1777,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1847,13 +1821,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1891,13 +1865,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1935,13 +1909,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1976,13 +1950,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2017,13 +1991,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2058,13 +2032,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2099,13 +2073,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2197,13 +2171,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2235,13 +2209,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2274,19 +2248,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (16/09/2026 12:40)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,8 +491,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -508,7 +516,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -516,12 +524,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -821,37 +847,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -901,58 +927,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -969,13 +995,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1010,13 +1036,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1051,13 +1077,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1092,13 +1118,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1133,13 +1159,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1177,13 +1203,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1218,13 +1244,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1259,13 +1285,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1297,13 +1323,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1338,13 +1364,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1379,13 +1405,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1417,13 +1443,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1455,13 +1481,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1496,13 +1522,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1537,13 +1563,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1578,13 +1604,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1619,13 +1645,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1660,13 +1686,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1701,13 +1727,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1736,13 +1762,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1777,13 +1803,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1821,13 +1847,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1865,13 +1891,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1909,13 +1935,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1950,13 +1976,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1991,13 +2017,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2032,13 +2058,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2073,13 +2099,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2171,13 +2197,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2209,13 +2235,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2248,19 +2274,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (17/09/2026 12:32)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="155">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -211,6 +211,9 @@
   </si>
   <si>
     <t>Módulo II – Orçamento 04/26</t>
+  </si>
+  <si>
+    <t>Módulo II – Orçamento 05/26</t>
   </si>
   <si>
     <t>Módulo III – Orçamento 17 Manuais</t>
@@ -491,16 +494,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -516,7 +511,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -524,30 +519,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -847,37 +824,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -923,62 +900,62 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R34"/>
+  <dimension ref="A1:R35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -990,34 +967,34 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
-        <v>70</v>
-      </c>
-      <c r="H2" s="2">
+        <v>71</v>
+      </c>
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
         <v>748504.24</v>
       </c>
       <c r="J2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K2">
         <v>748504.24</v>
       </c>
       <c r="M2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P2">
         <v>881914.1800000001</v>
@@ -1031,34 +1008,34 @@
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
-        <v>71</v>
-      </c>
-      <c r="H3" s="2">
+        <v>72</v>
+      </c>
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
         <v>1110378.24</v>
       </c>
       <c r="J3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K3">
         <v>1110378.24</v>
       </c>
       <c r="M3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P3">
         <v>2634000</v>
@@ -1072,34 +1049,34 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H4" s="2">
+        <v>73</v>
+      </c>
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
         <v>974557.12</v>
       </c>
       <c r="J4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K4">
         <v>974557.12</v>
       </c>
       <c r="M4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P4">
         <v>1686034.96</v>
@@ -1113,34 +1090,34 @@
         <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
-        <v>73</v>
-      </c>
-      <c r="H5" s="2">
+        <v>74</v>
+      </c>
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
         <v>1402001.34</v>
       </c>
       <c r="J5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K5">
         <v>1402001.34</v>
       </c>
       <c r="M5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P5">
         <v>1600334.09</v>
@@ -1154,34 +1131,34 @@
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
-        <v>74</v>
-      </c>
-      <c r="H6" s="2">
+        <v>75</v>
+      </c>
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
         <v>1223702.3</v>
       </c>
       <c r="J6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K6">
         <v>1223702.3</v>
       </c>
       <c r="M6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O6">
         <v>0.02</v>
@@ -1198,34 +1175,34 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
-        <v>75</v>
-      </c>
-      <c r="H7" s="2">
+        <v>76</v>
+      </c>
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
         <v>1011677.95</v>
       </c>
       <c r="J7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K7">
         <v>1011677.95</v>
       </c>
       <c r="M7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P7">
         <v>2568571.48</v>
@@ -1239,34 +1216,34 @@
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
-        <v>76</v>
-      </c>
-      <c r="H8" s="2">
+        <v>77</v>
+      </c>
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
         <v>896744.0600000001</v>
       </c>
       <c r="J8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K8">
         <v>896744.0600000001</v>
       </c>
       <c r="M8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P8">
         <v>968237.39</v>
@@ -1280,34 +1257,34 @@
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
-      </c>
-      <c r="H9" s="2">
+        <v>78</v>
+      </c>
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
         <v>919329.0600000001</v>
       </c>
       <c r="J9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K9">
         <v>919329.0600000001</v>
       </c>
       <c r="M9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P9">
         <v>1947932.74</v>
@@ -1323,29 +1300,29 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
-        <v>78</v>
-      </c>
-      <c r="H10" s="2">
+        <v>79</v>
+      </c>
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
         <v>1157009.26</v>
       </c>
       <c r="J10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K10">
         <v>1157009.26</v>
       </c>
       <c r="M10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P10">
         <v>3105605.8</v>
@@ -1359,34 +1336,34 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
-        <v>79</v>
-      </c>
-      <c r="H11" s="2">
+        <v>80</v>
+      </c>
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
         <v>1214597.952</v>
       </c>
       <c r="J11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K11">
         <v>1214597.952</v>
       </c>
       <c r="M11" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N11" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P11">
         <v>2096487.74</v>
@@ -1400,34 +1377,34 @@
         <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
-      </c>
-      <c r="H12" s="2">
+        <v>81</v>
+      </c>
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
         <v>967082.09</v>
       </c>
       <c r="J12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K12">
         <v>967082.09</v>
       </c>
       <c r="M12" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N12" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P12">
         <v>3522444.13</v>
@@ -1443,29 +1420,29 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
-      </c>
-      <c r="H13" s="2">
+        <v>82</v>
+      </c>
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
         <v>719561.08</v>
       </c>
       <c r="J13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K13">
         <v>719561.08</v>
       </c>
       <c r="M13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P13">
         <v>1500000</v>
@@ -1481,29 +1458,29 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
-        <v>82</v>
-      </c>
-      <c r="H14" s="2">
+        <v>83</v>
+      </c>
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
         <v>885881.08</v>
       </c>
       <c r="J14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K14">
         <v>885881.08</v>
       </c>
       <c r="M14" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N14" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O14">
         <v>34065.36</v>
@@ -1522,29 +1499,29 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
-        <v>83</v>
-      </c>
-      <c r="H15" s="2">
+        <v>84</v>
+      </c>
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
         <v>1350542.52</v>
       </c>
       <c r="J15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K15">
         <v>1350542.52</v>
       </c>
       <c r="M15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O15">
         <v>0.01</v>
@@ -1563,29 +1540,29 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
-        <v>84</v>
-      </c>
-      <c r="H16" s="2">
+        <v>85</v>
+      </c>
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
         <v>1108954.435833333</v>
       </c>
       <c r="J16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K16">
         <v>1108954.435833333</v>
       </c>
       <c r="M16" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N16" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O16">
         <v>0.01</v>
@@ -1604,29 +1581,29 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
-        <v>84</v>
-      </c>
-      <c r="H17" s="2">
+        <v>85</v>
+      </c>
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
         <v>218206.1</v>
       </c>
       <c r="J17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K17">
         <v>218206.1</v>
       </c>
       <c r="M17" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N17" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O17">
         <v>0.01</v>
@@ -1645,29 +1622,29 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
-        <v>84</v>
-      </c>
-      <c r="H18" s="2">
+        <v>85</v>
+      </c>
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
         <v>1549250.84</v>
       </c>
       <c r="J18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K18">
         <v>1549250.84</v>
       </c>
       <c r="M18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O18">
         <v>0.01</v>
@@ -1686,29 +1663,29 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
-        <v>85</v>
-      </c>
-      <c r="H19" s="2">
+        <v>86</v>
+      </c>
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
         <v>1340865.98</v>
       </c>
       <c r="J19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K19">
         <v>1340865.98</v>
       </c>
       <c r="M19" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N19" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O19">
         <v>927618.61</v>
@@ -1727,23 +1704,23 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
-        <v>86</v>
-      </c>
-      <c r="H20" s="2">
+        <v>87</v>
+      </c>
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
         <v>1629834.48</v>
       </c>
       <c r="M20" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N20" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O20">
         <v>282458.04</v>
@@ -1762,29 +1739,29 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
-        <v>87</v>
-      </c>
-      <c r="H21" s="2">
+        <v>88</v>
+      </c>
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
         <v>188246.17</v>
       </c>
       <c r="J21" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K21">
         <v>188246.17</v>
       </c>
       <c r="M21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P21">
         <v>211614.23</v>
@@ -1803,29 +1780,29 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
-        <v>88</v>
-      </c>
-      <c r="H22" s="2">
+        <v>89</v>
+      </c>
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
         <v>112720.77</v>
       </c>
       <c r="J22" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K22">
         <v>112720.77</v>
       </c>
       <c r="M22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N22" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O22">
         <v>0.01</v>
@@ -1842,34 +1819,34 @@
         <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
-        <v>89</v>
-      </c>
-      <c r="H23" s="2">
+        <v>90</v>
+      </c>
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
         <v>378307.61</v>
       </c>
       <c r="J23" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K23">
         <v>378307.61</v>
       </c>
       <c r="M23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O23">
         <v>0.01</v>
@@ -1886,34 +1863,34 @@
         <v>56</v>
       </c>
       <c r="C24" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
-        <v>89</v>
-      </c>
-      <c r="H24" s="2">
+        <v>90</v>
+      </c>
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
         <v>3315.047100000025</v>
       </c>
       <c r="J24" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K24">
         <v>3315.04710000003</v>
       </c>
       <c r="M24" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O24">
         <v>0.01</v>
@@ -1935,29 +1912,29 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
-        <v>73</v>
-      </c>
-      <c r="H25" s="2">
+        <v>74</v>
+      </c>
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
         <v>198332.75</v>
       </c>
       <c r="J25" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K25">
         <v>198332.75</v>
       </c>
       <c r="M25" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N25" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P25">
         <v>1600334.09</v>
@@ -1976,29 +1953,29 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H26" s="2">
+        <v>91</v>
+      </c>
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
         <v>1528.62</v>
       </c>
       <c r="J26" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K26">
         <v>1528.62</v>
       </c>
       <c r="M26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N26" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P26">
         <v>1157673.06</v>
@@ -2012,34 +1989,34 @@
         <v>59</v>
       </c>
       <c r="C27" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
-        <v>91</v>
-      </c>
-      <c r="H27" s="2">
+        <v>92</v>
+      </c>
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
         <v>38718.58</v>
       </c>
       <c r="J27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K27">
         <v>38718.58</v>
       </c>
       <c r="M27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P27">
         <v>63746.85</v>
@@ -2058,29 +2035,29 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
-        <v>92</v>
-      </c>
-      <c r="H28" s="2">
+        <v>93</v>
+      </c>
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
         <v>133124.11</v>
       </c>
       <c r="J28" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K28">
         <v>133124.11</v>
       </c>
       <c r="M28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P28">
         <v>1000001.64</v>
@@ -2099,29 +2076,29 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
-        <v>81</v>
-      </c>
-      <c r="H29" s="2">
+        <v>82</v>
+      </c>
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
         <v>11372.9</v>
       </c>
       <c r="J29" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K29">
         <v>11372.9</v>
       </c>
       <c r="M29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P29">
         <v>1500000</v>
@@ -2135,16 +2112,16 @@
         <v>62</v>
       </c>
       <c r="G30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L30">
         <v>15854.78</v>
       </c>
       <c r="M30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -2155,16 +2132,16 @@
         <v>63</v>
       </c>
       <c r="G31" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L31">
         <v>42229.72325</v>
       </c>
       <c r="M31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -2175,54 +2152,36 @@
         <v>64</v>
       </c>
       <c r="G32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L32">
         <v>48857.39550000001</v>
       </c>
       <c r="M32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:16">
       <c r="A33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="D33">
-        <v>1465</v>
-      </c>
-      <c r="E33" s="2">
-        <v>46104</v>
-      </c>
-      <c r="F33" t="s">
-        <v>81</v>
-      </c>
-      <c r="H33" s="2">
-        <v>46106</v>
-      </c>
-      <c r="I33">
-        <v>27801.11</v>
-      </c>
-      <c r="J33" t="s">
-        <v>121</v>
-      </c>
-      <c r="K33">
-        <v>27801.11</v>
+      <c r="G33" t="s">
+        <v>95</v>
+      </c>
+      <c r="L33">
+        <v>4192.68</v>
       </c>
       <c r="M33" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N33" t="s">
-        <v>125</v>
-      </c>
-      <c r="P33">
-        <v>1500000</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:16">
@@ -2233,33 +2192,71 @@
         <v>66</v>
       </c>
       <c r="D34">
-        <v>1882</v>
-      </c>
-      <c r="E34" s="2">
-        <v>46199</v>
+        <v>1465</v>
+      </c>
+      <c r="E34" s="1">
+        <v>46104</v>
       </c>
       <c r="F34" t="s">
-        <v>93</v>
-      </c>
-      <c r="H34" s="2">
-        <v>46233</v>
+        <v>82</v>
+      </c>
+      <c r="H34" s="1">
+        <v>46106</v>
       </c>
       <c r="I34">
-        <v>58868.35</v>
+        <v>27801.11</v>
       </c>
       <c r="J34" t="s">
         <v>122</v>
       </c>
       <c r="K34">
+        <v>27801.11</v>
+      </c>
+      <c r="M34" t="s">
+        <v>125</v>
+      </c>
+      <c r="N34" t="s">
+        <v>126</v>
+      </c>
+      <c r="P34">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16">
+      <c r="A35">
+        <v>3</v>
+      </c>
+      <c r="B35" t="s">
+        <v>67</v>
+      </c>
+      <c r="D35">
+        <v>1882</v>
+      </c>
+      <c r="E35" s="1">
+        <v>46199</v>
+      </c>
+      <c r="F35" t="s">
+        <v>94</v>
+      </c>
+      <c r="H35" s="1">
+        <v>46233</v>
+      </c>
+      <c r="I35">
         <v>58868.35</v>
       </c>
-      <c r="M34" t="s">
-        <v>124</v>
-      </c>
-      <c r="N34" t="s">
-        <v>126</v>
-      </c>
-      <c r="P34">
+      <c r="J35" t="s">
+        <v>123</v>
+      </c>
+      <c r="K35">
+        <v>58868.35</v>
+      </c>
+      <c r="M35" t="s">
+        <v>125</v>
+      </c>
+      <c r="N35" t="s">
+        <v>127</v>
+      </c>
+      <c r="P35">
         <v>2364771.07</v>
       </c>
     </row>
@@ -2274,25 +2271,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" t="s">
         <v>131</v>
+      </c>
+      <c r="E1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B2">
         <v>1000</v>
@@ -2303,7 +2300,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B3">
         <v>52250.04</v>
@@ -2314,7 +2311,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B4">
         <v>881914.1800000001</v>
@@ -2325,7 +2322,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B5">
         <v>750000</v>
@@ -2336,7 +2333,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B6">
         <v>949835.78</v>
@@ -2347,7 +2344,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B7">
         <v>524584.95</v>
@@ -2358,7 +2355,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B8">
         <v>211614.23</v>
@@ -2369,7 +2366,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B9">
         <v>2391157.41</v>
@@ -2380,7 +2377,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B10">
         <v>618154.38</v>
@@ -2391,7 +2388,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B11">
         <v>1600334.09</v>
@@ -2402,7 +2399,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B12">
         <v>2364771.07</v>
@@ -2413,7 +2410,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B13">
         <v>968237.39</v>
@@ -2424,7 +2421,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B14">
         <v>1011677.95</v>
@@ -2435,7 +2432,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B15">
         <v>1580293.02</v>
@@ -2446,7 +2443,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2457,7 +2454,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B17">
         <v>63746.85</v>
@@ -2468,7 +2465,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B18">
         <v>947931.1</v>
@@ -2479,7 +2476,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B19">
         <v>259790.57</v>
@@ -2490,7 +2487,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B20">
         <v>170479.3</v>
@@ -2501,7 +2498,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B21">
         <v>1500000</v>
@@ -2512,7 +2509,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B22">
         <v>1000001.64</v>
@@ -2523,7 +2520,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B23">
         <v>68405.66</v>
@@ -2534,7 +2531,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B24">
         <v>1157673.06</v>
@@ -2545,7 +2542,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B25">
         <v>34065.36</v>
@@ -2556,7 +2553,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B26">
         <v>843261.89</v>
@@ -2567,7 +2564,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B27">
         <v>1629834.48</v>
@@ -2578,7 +2575,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -2589,7 +2586,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -2600,7 +2597,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -2611,7 +2608,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B31">
         <v>0</v>
@@ -2622,7 +2619,7 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B32">
         <v>0</v>
@@ -2633,7 +2630,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B33">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (17/09/2026 12:58)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="156">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -485,6 +485,9 @@
   </si>
   <si>
     <t>2026NE001015</t>
+  </si>
+  <si>
+    <t>2026NE901182</t>
   </si>
 </sst>
 </file>
@@ -494,8 +497,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -511,7 +522,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -519,12 +530,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -824,37 +853,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -904,58 +933,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -972,13 +1001,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1013,13 +1042,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1054,13 +1083,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>73</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1095,13 +1124,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1136,13 +1165,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1180,13 +1209,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1221,13 +1250,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1262,13 +1291,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1300,13 +1329,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1341,13 +1370,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1382,13 +1411,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>81</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1406,8 +1435,11 @@
       <c r="N12" t="s">
         <v>126</v>
       </c>
+      <c r="O12">
+        <v>0.01</v>
+      </c>
       <c r="P12">
-        <v>3522444.13</v>
+        <v>3522444.12</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -1420,13 +1452,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1458,13 +1490,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1483,10 +1515,10 @@
         <v>126</v>
       </c>
       <c r="O14">
-        <v>34065.36</v>
+        <v>34065.35</v>
       </c>
       <c r="P14">
-        <v>3080293.02</v>
+        <v>3080293.03</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -1499,13 +1531,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1540,13 +1572,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>85</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1565,10 +1597,10 @@
         <v>126</v>
       </c>
       <c r="O16">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="P16">
-        <v>6336221.5</v>
+        <v>6336221.49</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -1581,13 +1613,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1606,10 +1638,10 @@
         <v>126</v>
       </c>
       <c r="O17">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="P17">
-        <v>6336221.5</v>
+        <v>6336221.49</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -1622,13 +1654,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>85</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1647,10 +1679,10 @@
         <v>126</v>
       </c>
       <c r="O18">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="P18">
-        <v>6336221.5</v>
+        <v>6336221.49</v>
       </c>
     </row>
     <row r="19" spans="1:16">
@@ -1663,13 +1695,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>86</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1688,10 +1720,10 @@
         <v>126</v>
       </c>
       <c r="O19">
-        <v>927618.61</v>
+        <v>927618.62</v>
       </c>
       <c r="P19">
-        <v>3208032.96</v>
+        <v>3208032.95</v>
       </c>
     </row>
     <row r="20" spans="1:16">
@@ -1704,13 +1736,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1739,13 +1771,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>88</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1780,13 +1812,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>89</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1824,13 +1856,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>90</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1868,13 +1900,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>90</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1912,13 +1944,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>74</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1953,13 +1985,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>91</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1994,13 +2026,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>92</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2035,13 +2067,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>93</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2076,13 +2108,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>82</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2194,13 +2226,13 @@
       <c r="D34">
         <v>1465</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46104</v>
       </c>
       <c r="F34" t="s">
         <v>82</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46106</v>
       </c>
       <c r="I34">
@@ -2232,13 +2264,13 @@
       <c r="D35">
         <v>1882</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46199</v>
       </c>
       <c r="F35" t="s">
         <v>94</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46233</v>
       </c>
       <c r="I35">
@@ -2256,8 +2288,11 @@
       <c r="N35" t="s">
         <v>127</v>
       </c>
+      <c r="O35">
+        <v>0.01</v>
+      </c>
       <c r="P35">
-        <v>2364771.07</v>
+        <v>2364771.06</v>
       </c>
     </row>
   </sheetData>
@@ -2267,23 +2302,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>132</v>
       </c>
     </row>
@@ -2402,10 +2437,10 @@
         <v>94</v>
       </c>
       <c r="B12">
-        <v>2364771.07</v>
+        <v>2364771.06</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -2446,10 +2481,10 @@
         <v>142</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="C16">
-        <v>34065.36</v>
+        <v>34065.35</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -2637,6 +2672,17 @@
       </c>
       <c r="C33">
         <v>236343.68</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>155</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="C34">
+        <v>1145462.93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (18/09/2026 11:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -497,16 +497,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -522,7 +514,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -530,30 +522,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -853,37 +827,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -933,58 +907,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1001,13 +975,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1042,13 +1016,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1083,13 +1057,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>73</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1124,13 +1098,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1165,13 +1139,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1209,13 +1183,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1250,13 +1224,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1291,13 +1265,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1329,13 +1303,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1370,13 +1344,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1411,13 +1385,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>81</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1452,13 +1426,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1490,13 +1464,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1531,13 +1505,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1572,13 +1546,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>85</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1613,13 +1587,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1654,13 +1628,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>85</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1695,13 +1669,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>86</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1736,13 +1710,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1771,13 +1745,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>88</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1812,13 +1786,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>89</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1856,13 +1830,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>90</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1900,13 +1874,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>90</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1944,13 +1918,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>74</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1985,13 +1959,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>91</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2026,13 +2000,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>92</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2067,13 +2041,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>93</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2108,13 +2082,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>82</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2226,13 +2200,13 @@
       <c r="D34">
         <v>1465</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46104</v>
       </c>
       <c r="F34" t="s">
         <v>82</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46106</v>
       </c>
       <c r="I34">
@@ -2264,13 +2238,13 @@
       <c r="D35">
         <v>1882</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>46199</v>
       </c>
       <c r="F35" t="s">
         <v>94</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46233</v>
       </c>
       <c r="I35">
@@ -2306,19 +2280,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>132</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (18/09/2026 16:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -497,8 +497,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -514,7 +522,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -522,12 +530,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -827,37 +853,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -907,58 +933,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -975,13 +1001,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1016,13 +1042,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1057,13 +1083,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>73</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1098,13 +1124,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1139,13 +1165,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1183,13 +1209,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1224,13 +1250,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1265,13 +1291,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1303,13 +1329,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1344,13 +1370,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1385,13 +1411,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>81</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1426,13 +1452,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1464,13 +1490,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1505,13 +1531,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1546,13 +1572,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>85</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1587,13 +1613,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1628,13 +1654,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>85</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1669,13 +1695,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>86</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1710,13 +1736,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1745,13 +1771,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>88</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1786,13 +1812,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>89</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1830,13 +1856,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>90</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1874,13 +1900,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>90</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1918,13 +1944,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>74</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1959,13 +1985,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>91</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2000,13 +2026,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>92</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2041,13 +2067,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>93</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2082,13 +2108,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>82</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2200,13 +2226,13 @@
       <c r="D34">
         <v>1465</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46104</v>
       </c>
       <c r="F34" t="s">
         <v>82</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46106</v>
       </c>
       <c r="I34">
@@ -2238,13 +2264,13 @@
       <c r="D35">
         <v>1882</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46199</v>
       </c>
       <c r="F35" t="s">
         <v>94</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46233</v>
       </c>
       <c r="I35">
@@ -2280,19 +2306,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>132</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (21/09/2026 14:30)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -497,8 +497,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -514,7 +522,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -522,12 +530,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -827,37 +853,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -907,58 +933,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -975,13 +1001,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1016,13 +1042,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1057,13 +1083,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>73</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1098,13 +1124,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1139,13 +1165,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1183,13 +1209,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1224,13 +1250,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1265,13 +1291,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1303,13 +1329,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1344,13 +1370,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1385,13 +1411,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>81</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1426,13 +1452,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1464,13 +1490,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1505,13 +1531,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1546,13 +1572,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>85</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1587,13 +1613,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1628,13 +1654,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>85</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1669,13 +1695,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>86</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1710,13 +1736,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1745,13 +1771,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>88</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1786,13 +1812,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>89</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1830,13 +1856,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>90</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1874,13 +1900,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>90</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1918,13 +1944,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>74</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1959,13 +1985,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>91</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2000,13 +2026,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>92</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2041,13 +2067,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>93</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2082,13 +2108,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>82</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2200,13 +2226,13 @@
       <c r="D34">
         <v>1465</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46104</v>
       </c>
       <c r="F34" t="s">
         <v>82</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46106</v>
       </c>
       <c r="I34">
@@ -2238,13 +2264,13 @@
       <c r="D35">
         <v>1882</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46199</v>
       </c>
       <c r="F35" t="s">
         <v>94</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46233</v>
       </c>
       <c r="I35">
@@ -2280,19 +2306,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>132</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (22/09/2026 12:30)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -497,16 +497,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -522,7 +514,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -530,30 +522,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -853,37 +827,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -933,58 +907,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1001,13 +975,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1042,13 +1016,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1083,13 +1057,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>73</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1124,13 +1098,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1165,13 +1139,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1209,13 +1183,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1250,13 +1224,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1291,13 +1265,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1329,13 +1303,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1370,13 +1344,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1411,13 +1385,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>81</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1452,13 +1426,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1490,13 +1464,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1531,13 +1505,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1572,13 +1546,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>85</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1613,13 +1587,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1654,13 +1628,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>85</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1695,13 +1669,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>86</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1736,13 +1710,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1771,13 +1745,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>88</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1812,13 +1786,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>89</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1856,13 +1830,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>90</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1900,13 +1874,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>90</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1944,13 +1918,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>74</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1985,13 +1959,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>91</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2026,13 +2000,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>92</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2067,13 +2041,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>93</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2108,13 +2082,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>82</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2226,13 +2200,13 @@
       <c r="D34">
         <v>1465</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46104</v>
       </c>
       <c r="F34" t="s">
         <v>82</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46106</v>
       </c>
       <c r="I34">
@@ -2264,13 +2238,13 @@
       <c r="D35">
         <v>1882</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>46199</v>
       </c>
       <c r="F35" t="s">
         <v>94</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46233</v>
       </c>
       <c r="I35">
@@ -2306,19 +2280,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>132</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (23/09/2026 10:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -497,8 +497,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -514,7 +522,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -522,12 +530,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -827,37 +853,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -907,58 +933,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -975,13 +1001,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1016,13 +1042,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1057,13 +1083,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>73</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1098,13 +1124,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1139,13 +1165,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1183,13 +1209,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1224,13 +1250,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1265,13 +1291,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1303,13 +1329,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1344,13 +1370,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1385,13 +1411,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>81</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1426,13 +1452,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1464,13 +1490,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1505,13 +1531,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1546,13 +1572,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>85</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1587,13 +1613,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1628,13 +1654,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>85</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1669,13 +1695,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>86</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1710,13 +1736,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1745,13 +1771,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>88</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1786,13 +1812,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>89</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1830,13 +1856,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>90</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1874,13 +1900,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>90</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1918,13 +1944,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>74</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1959,13 +1985,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>91</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2000,13 +2026,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>92</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2041,13 +2067,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>93</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2082,13 +2108,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>82</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2200,13 +2226,13 @@
       <c r="D34">
         <v>1465</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46104</v>
       </c>
       <c r="F34" t="s">
         <v>82</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46106</v>
       </c>
       <c r="I34">
@@ -2238,13 +2264,13 @@
       <c r="D35">
         <v>1882</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46199</v>
       </c>
       <c r="F35" t="s">
         <v>94</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46233</v>
       </c>
       <c r="I35">
@@ -2280,19 +2306,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>132</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (23/09/2026 12:26)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -497,16 +497,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -522,7 +514,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -530,30 +522,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -853,37 +827,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -933,58 +907,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1001,13 +975,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1042,13 +1016,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1083,13 +1057,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>73</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1124,13 +1098,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1165,13 +1139,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1209,13 +1183,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1250,13 +1224,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1291,13 +1265,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1329,13 +1303,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1370,13 +1344,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1411,13 +1385,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>81</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1452,13 +1426,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1490,13 +1464,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1531,13 +1505,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1572,13 +1546,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>85</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1613,13 +1587,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1654,13 +1628,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>85</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1695,13 +1669,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>86</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1736,13 +1710,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1771,13 +1745,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>88</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1812,13 +1786,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>89</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1856,13 +1830,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>90</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1900,13 +1874,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>90</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1944,13 +1918,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>74</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1985,13 +1959,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>91</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2026,13 +2000,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>92</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2067,13 +2041,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>93</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2108,13 +2082,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>82</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2226,13 +2200,13 @@
       <c r="D34">
         <v>1465</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46104</v>
       </c>
       <c r="F34" t="s">
         <v>82</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46106</v>
       </c>
       <c r="I34">
@@ -2264,13 +2238,13 @@
       <c r="D35">
         <v>1882</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>46199</v>
       </c>
       <c r="F35" t="s">
         <v>94</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46233</v>
       </c>
       <c r="I35">
@@ -2306,19 +2280,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>132</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (28/09/2026 13:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -497,8 +497,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -514,7 +522,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -522,12 +530,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -827,37 +853,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -907,58 +933,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -975,13 +1001,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1016,13 +1042,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1057,13 +1083,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>73</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1098,13 +1124,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1139,13 +1165,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1183,13 +1209,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1224,13 +1250,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1265,13 +1291,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1303,13 +1329,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1344,13 +1370,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1385,13 +1411,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>81</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1426,13 +1452,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1464,13 +1490,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1505,13 +1531,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1546,13 +1572,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>85</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1587,13 +1613,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1628,13 +1654,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>85</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1669,13 +1695,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>86</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1710,13 +1736,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1745,13 +1771,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>88</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1786,13 +1812,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>89</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1830,13 +1856,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>90</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1874,13 +1900,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>90</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1918,13 +1944,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>74</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1959,13 +1985,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>91</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2000,13 +2026,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>92</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2041,13 +2067,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>93</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2082,13 +2108,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>82</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2200,13 +2226,13 @@
       <c r="D34">
         <v>1465</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46104</v>
       </c>
       <c r="F34" t="s">
         <v>82</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46106</v>
       </c>
       <c r="I34">
@@ -2238,13 +2264,13 @@
       <c r="D35">
         <v>1882</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46199</v>
       </c>
       <c r="F35" t="s">
         <v>94</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46233</v>
       </c>
       <c r="I35">
@@ -2280,19 +2306,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>132</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (28/09/2026 13:14)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="160">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -175,6 +175,9 @@
   </si>
   <si>
     <t>JULHO/26</t>
+  </si>
+  <si>
+    <t>AGOSTO/26</t>
   </si>
   <si>
     <t>Módulo II – Parcial Orçamento 10 (FAB 2728)</t>
@@ -286,6 +289,9 @@
     <t>2026NE000388</t>
   </si>
   <si>
+    <t>2026NE000330, 2026NE000388, 2026NE000816, 2026NE000817, 2026NE001015</t>
+  </si>
+  <si>
     <t>2025NE000559</t>
   </si>
   <si>
@@ -361,6 +367,12 @@
     <t>2026NP402899</t>
   </si>
   <si>
+    <t>2026NP403306</t>
+  </si>
+  <si>
+    <t>2026NP403583</t>
+  </si>
+  <si>
     <t>2025NP002620</t>
   </si>
   <si>
@@ -403,10 +415,10 @@
     <t>Pago</t>
   </si>
   <si>
+    <t>Pendente</t>
+  </si>
+  <si>
     <t>Faturado, aguardando pagamento</t>
-  </si>
-  <si>
-    <t>Pendente</t>
   </si>
   <si>
     <t>numero_empenho</t>
@@ -929,7 +941,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R35"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
@@ -996,7 +1008,7 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D2">
         <v>594</v>
@@ -1005,7 +1017,7 @@
         <v>45740</v>
       </c>
       <c r="F2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H2" s="2">
         <v>45778</v>
@@ -1014,16 +1026,16 @@
         <v>748504.24</v>
       </c>
       <c r="J2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K2">
         <v>748504.24</v>
       </c>
       <c r="M2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P2">
         <v>881914.1800000001</v>
@@ -1037,7 +1049,7 @@
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D3">
         <v>620</v>
@@ -1046,7 +1058,7 @@
         <v>45775</v>
       </c>
       <c r="F3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H3" s="2">
         <v>45806</v>
@@ -1055,16 +1067,16 @@
         <v>1110378.24</v>
       </c>
       <c r="J3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="K3">
         <v>1110378.24</v>
       </c>
       <c r="M3" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N3" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P3">
         <v>2634000</v>
@@ -1078,7 +1090,7 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D4">
         <v>634</v>
@@ -1087,7 +1099,7 @@
         <v>45799</v>
       </c>
       <c r="F4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H4" s="2">
         <v>45844</v>
@@ -1096,16 +1108,16 @@
         <v>974557.12</v>
       </c>
       <c r="J4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K4">
         <v>974557.12</v>
       </c>
       <c r="M4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P4">
         <v>1686034.96</v>
@@ -1119,7 +1131,7 @@
         <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D5">
         <v>660</v>
@@ -1128,7 +1140,7 @@
         <v>45856</v>
       </c>
       <c r="F5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H5" s="2">
         <v>45891</v>
@@ -1137,16 +1149,16 @@
         <v>1402001.34</v>
       </c>
       <c r="J5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K5">
         <v>1402001.34</v>
       </c>
       <c r="M5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P5">
         <v>1600334.09</v>
@@ -1160,7 +1172,7 @@
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D6">
         <v>661</v>
@@ -1169,7 +1181,7 @@
         <v>45856</v>
       </c>
       <c r="F6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H6" s="2">
         <v>45891</v>
@@ -1178,16 +1190,16 @@
         <v>1223702.3</v>
       </c>
       <c r="J6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K6">
         <v>1223702.3</v>
       </c>
       <c r="M6" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N6" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="O6">
         <v>0.02</v>
@@ -1204,7 +1216,7 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D7">
         <v>688</v>
@@ -1213,7 +1225,7 @@
         <v>45901</v>
       </c>
       <c r="F7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H7" s="2">
         <v>45938</v>
@@ -1222,16 +1234,16 @@
         <v>1011677.95</v>
       </c>
       <c r="J7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="K7">
         <v>1011677.95</v>
       </c>
       <c r="M7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P7">
         <v>2568571.48</v>
@@ -1245,7 +1257,7 @@
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D8">
         <v>696</v>
@@ -1254,7 +1266,7 @@
         <v>45923</v>
       </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H8" s="2">
         <v>45938</v>
@@ -1263,16 +1275,16 @@
         <v>896744.0600000001</v>
       </c>
       <c r="J8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K8">
         <v>896744.0600000001</v>
       </c>
       <c r="M8" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N8" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P8">
         <v>968237.39</v>
@@ -1286,7 +1298,7 @@
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D9">
         <v>704</v>
@@ -1295,7 +1307,7 @@
         <v>45957</v>
       </c>
       <c r="F9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H9" s="2">
         <v>46003</v>
@@ -1304,16 +1316,16 @@
         <v>919329.0600000001</v>
       </c>
       <c r="J9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="K9">
         <v>919329.0600000001</v>
       </c>
       <c r="M9" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N9" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P9">
         <v>1947932.74</v>
@@ -1333,7 +1345,7 @@
         <v>45972</v>
       </c>
       <c r="F10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H10" s="2">
         <v>46016</v>
@@ -1342,16 +1354,16 @@
         <v>1157009.26</v>
       </c>
       <c r="J10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K10">
         <v>1157009.26</v>
       </c>
       <c r="M10" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N10" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P10">
         <v>3105605.8</v>
@@ -1365,7 +1377,7 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D11">
         <v>728</v>
@@ -1374,7 +1386,7 @@
         <v>46008</v>
       </c>
       <c r="F11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H11" s="2">
         <v>46040</v>
@@ -1383,16 +1395,16 @@
         <v>1214597.952</v>
       </c>
       <c r="J11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="K11">
         <v>1214597.952</v>
       </c>
       <c r="M11" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N11" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P11">
         <v>2096487.74</v>
@@ -1406,7 +1418,7 @@
         <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D12">
         <v>278</v>
@@ -1415,7 +1427,7 @@
         <v>46042</v>
       </c>
       <c r="F12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H12" s="2">
         <v>46074</v>
@@ -1424,16 +1436,16 @@
         <v>967082.09</v>
       </c>
       <c r="J12" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K12">
         <v>967082.09</v>
       </c>
       <c r="M12" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N12" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="O12">
         <v>0.01</v>
@@ -1456,7 +1468,7 @@
         <v>46078</v>
       </c>
       <c r="F13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H13" s="2">
         <v>46106</v>
@@ -1465,16 +1477,16 @@
         <v>719561.08</v>
       </c>
       <c r="J13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K13">
         <v>719561.08</v>
       </c>
       <c r="M13" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N13" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P13">
         <v>1500000</v>
@@ -1494,7 +1506,7 @@
         <v>46094</v>
       </c>
       <c r="F14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H14" s="2">
         <v>46128</v>
@@ -1503,16 +1515,16 @@
         <v>885881.08</v>
       </c>
       <c r="J14" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K14">
         <v>885881.08</v>
       </c>
       <c r="M14" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N14" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="O14">
         <v>34065.35</v>
@@ -1535,7 +1547,7 @@
         <v>46128</v>
       </c>
       <c r="F15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H15" s="2">
         <v>46164</v>
@@ -1544,16 +1556,16 @@
         <v>1350542.52</v>
       </c>
       <c r="J15" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="K15">
         <v>1350542.52</v>
       </c>
       <c r="M15" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N15" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="O15">
         <v>0.01</v>
@@ -1576,7 +1588,7 @@
         <v>46156</v>
       </c>
       <c r="F16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H16" s="2">
         <v>46191</v>
@@ -1585,16 +1597,16 @@
         <v>1108954.435833333</v>
       </c>
       <c r="J16" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K16">
         <v>1108954.435833333</v>
       </c>
       <c r="M16" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N16" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="O16">
         <v>0.02</v>
@@ -1617,7 +1629,7 @@
         <v>46149</v>
       </c>
       <c r="F17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H17" s="2">
         <v>46185</v>
@@ -1626,16 +1638,16 @@
         <v>218206.1</v>
       </c>
       <c r="J17" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K17">
         <v>218206.1</v>
       </c>
       <c r="M17" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N17" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="O17">
         <v>0.02</v>
@@ -1658,7 +1670,7 @@
         <v>46156</v>
       </c>
       <c r="F18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H18" s="2">
         <v>46191</v>
@@ -1667,16 +1679,16 @@
         <v>1549250.84</v>
       </c>
       <c r="J18" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="K18">
         <v>1549250.84</v>
       </c>
       <c r="M18" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N18" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="O18">
         <v>0.02</v>
@@ -1699,7 +1711,7 @@
         <v>46230</v>
       </c>
       <c r="F19" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H19" s="2">
         <v>46262</v>
@@ -1708,16 +1720,16 @@
         <v>1340865.98</v>
       </c>
       <c r="J19" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K19">
         <v>1340865.98</v>
       </c>
       <c r="M19" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N19" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="O19">
         <v>927618.62</v>
@@ -1740,19 +1752,25 @@
         <v>46252</v>
       </c>
       <c r="F20" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H20" s="2">
         <v>46284</v>
       </c>
+      <c r="I20">
+        <v>1629834.48</v>
+      </c>
+      <c r="J20" t="s">
+        <v>115</v>
+      </c>
       <c r="K20">
         <v>1629834.48</v>
       </c>
       <c r="M20" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N20" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="O20">
         <v>282458.04</v>
@@ -1763,40 +1781,43 @@
     </row>
     <row r="21" spans="1:16">
       <c r="A21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B21" t="s">
         <v>53</v>
       </c>
       <c r="D21">
-        <v>402</v>
+        <v>66</v>
       </c>
       <c r="E21" s="2">
-        <v>45791</v>
+        <v>46280</v>
       </c>
       <c r="F21" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H21" s="2">
-        <v>45834</v>
+        <v>46312</v>
       </c>
       <c r="I21">
-        <v>188246.17</v>
+        <v>1675964.21</v>
       </c>
       <c r="J21" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="K21">
-        <v>188246.17</v>
+        <v>1675964.21</v>
       </c>
       <c r="M21" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="N21" t="s">
-        <v>126</v>
+        <v>130</v>
+      </c>
+      <c r="O21">
+        <v>2089048.83</v>
       </c>
       <c r="P21">
-        <v>211614.23</v>
+        <v>2473096.37</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -1806,41 +1827,35 @@
       <c r="B22" t="s">
         <v>54</v>
       </c>
-      <c r="C22">
-        <v>46</v>
-      </c>
       <c r="D22">
-        <v>447</v>
+        <v>402</v>
       </c>
       <c r="E22" s="2">
-        <v>45814</v>
+        <v>45791</v>
       </c>
       <c r="F22" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H22" s="2">
-        <v>45955</v>
+        <v>45834</v>
       </c>
       <c r="I22">
-        <v>112720.77</v>
+        <v>188246.17</v>
       </c>
       <c r="J22" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="K22">
-        <v>112720.77</v>
+        <v>188246.17</v>
       </c>
       <c r="M22" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N22" t="s">
-        <v>126</v>
-      </c>
-      <c r="O22">
-        <v>0.01</v>
+        <v>130</v>
       </c>
       <c r="P22">
-        <v>3359394.8</v>
+        <v>211614.23</v>
       </c>
     </row>
     <row r="23" spans="1:16">
@@ -1850,41 +1865,41 @@
       <c r="B23" t="s">
         <v>55</v>
       </c>
-      <c r="C23" t="s">
-        <v>69</v>
+      <c r="C23">
+        <v>46</v>
       </c>
       <c r="D23">
-        <v>529</v>
+        <v>447</v>
       </c>
       <c r="E23" s="2">
-        <v>45853</v>
+        <v>45814</v>
       </c>
       <c r="F23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H23" s="2">
-        <v>45939</v>
+        <v>45955</v>
       </c>
       <c r="I23">
-        <v>378307.61</v>
+        <v>112720.77</v>
       </c>
       <c r="J23" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="K23">
-        <v>378307.61</v>
+        <v>112720.77</v>
       </c>
       <c r="M23" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N23" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="O23">
         <v>0.01</v>
       </c>
       <c r="P23">
-        <v>2391157.41</v>
+        <v>3359394.8</v>
       </c>
     </row>
     <row r="24" spans="1:16">
@@ -1895,34 +1910,34 @@
         <v>56</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D24">
-        <v>691</v>
+        <v>529</v>
       </c>
       <c r="E24" s="2">
-        <v>45910</v>
+        <v>45853</v>
       </c>
       <c r="F24" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H24" s="2">
-        <v>45941</v>
+        <v>45939</v>
       </c>
       <c r="I24">
-        <v>3315.047100000025</v>
+        <v>378307.61</v>
       </c>
       <c r="J24" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="K24">
-        <v>3315.04710000003</v>
+        <v>378307.61</v>
       </c>
       <c r="M24" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N24" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="O24">
         <v>0.01</v>
@@ -1938,38 +1953,41 @@
       <c r="B25" t="s">
         <v>57</v>
       </c>
-      <c r="C25">
-        <v>135</v>
+      <c r="C25" t="s">
+        <v>70</v>
       </c>
       <c r="D25">
-        <v>677</v>
+        <v>691</v>
       </c>
       <c r="E25" s="2">
-        <v>45904</v>
+        <v>45910</v>
       </c>
       <c r="F25" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="H25" s="2">
-        <v>45935</v>
+        <v>45941</v>
       </c>
       <c r="I25">
-        <v>198332.75</v>
+        <v>3315.047100000025</v>
       </c>
       <c r="J25" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="K25">
-        <v>198332.75</v>
+        <v>3315.04710000003</v>
       </c>
       <c r="M25" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N25" t="s">
-        <v>126</v>
+        <v>130</v>
+      </c>
+      <c r="O25">
+        <v>0.01</v>
       </c>
       <c r="P25">
-        <v>1600334.09</v>
+        <v>2391157.41</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -1980,37 +1998,37 @@
         <v>58</v>
       </c>
       <c r="C26">
-        <v>40</v>
+        <v>135</v>
       </c>
       <c r="D26">
-        <v>278</v>
+        <v>677</v>
       </c>
       <c r="E26" s="2">
-        <v>46008</v>
+        <v>45904</v>
       </c>
       <c r="F26" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="H26" s="2">
-        <v>46066</v>
+        <v>45935</v>
       </c>
       <c r="I26">
-        <v>1528.62</v>
+        <v>198332.75</v>
       </c>
       <c r="J26" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="K26">
-        <v>1528.62</v>
+        <v>198332.75</v>
       </c>
       <c r="M26" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N26" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P26">
-        <v>1157673.06</v>
+        <v>1600334.09</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -2020,38 +2038,38 @@
       <c r="B27" t="s">
         <v>59</v>
       </c>
-      <c r="C27" t="s">
-        <v>70</v>
+      <c r="C27">
+        <v>40</v>
       </c>
       <c r="D27">
-        <v>748</v>
+        <v>278</v>
       </c>
       <c r="E27" s="2">
-        <v>45930</v>
+        <v>46008</v>
       </c>
       <c r="F27" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H27" s="2">
-        <v>45935</v>
+        <v>46066</v>
       </c>
       <c r="I27">
-        <v>38718.58</v>
+        <v>1528.62</v>
       </c>
       <c r="J27" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="K27">
-        <v>38718.58</v>
+        <v>1528.62</v>
       </c>
       <c r="M27" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N27" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P27">
-        <v>63746.85</v>
+        <v>1157673.06</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -2061,38 +2079,38 @@
       <c r="B28" t="s">
         <v>60</v>
       </c>
-      <c r="C28">
-        <v>154</v>
+      <c r="C28" t="s">
+        <v>71</v>
       </c>
       <c r="D28">
-        <v>822</v>
+        <v>748</v>
       </c>
       <c r="E28" s="2">
-        <v>45968</v>
+        <v>45930</v>
       </c>
       <c r="F28" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
-        <v>133124.11</v>
+        <v>38718.58</v>
       </c>
       <c r="J28" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="K28">
-        <v>133124.11</v>
+        <v>38718.58</v>
       </c>
       <c r="M28" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N28" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P28">
-        <v>1000001.64</v>
+        <v>63746.85</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -2103,37 +2121,37 @@
         <v>61</v>
       </c>
       <c r="C29">
-        <v>252</v>
+        <v>154</v>
       </c>
       <c r="D29">
-        <v>360</v>
+        <v>822</v>
       </c>
       <c r="E29" s="2">
-        <v>46043</v>
+        <v>45968</v>
       </c>
       <c r="F29" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H29" s="2">
-        <v>46075</v>
+        <v>45935</v>
       </c>
       <c r="I29">
-        <v>11372.9</v>
+        <v>133124.11</v>
       </c>
       <c r="J29" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="K29">
-        <v>11372.9</v>
+        <v>133124.11</v>
       </c>
       <c r="M29" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N29" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P29">
-        <v>1500000</v>
+        <v>1000001.64</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -2143,17 +2161,38 @@
       <c r="B30" t="s">
         <v>62</v>
       </c>
-      <c r="G30" t="s">
-        <v>95</v>
-      </c>
-      <c r="L30">
-        <v>15854.78</v>
+      <c r="C30">
+        <v>252</v>
+      </c>
+      <c r="D30">
+        <v>360</v>
+      </c>
+      <c r="E30" s="2">
+        <v>46043</v>
+      </c>
+      <c r="F30" t="s">
+        <v>83</v>
+      </c>
+      <c r="H30" s="2">
+        <v>46075</v>
+      </c>
+      <c r="I30">
+        <v>11372.9</v>
+      </c>
+      <c r="J30" t="s">
+        <v>125</v>
+      </c>
+      <c r="K30">
+        <v>11372.9</v>
       </c>
       <c r="M30" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N30" t="s">
-        <v>128</v>
+        <v>130</v>
+      </c>
+      <c r="P30">
+        <v>1500000</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -2164,16 +2203,16 @@
         <v>63</v>
       </c>
       <c r="G31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L31">
-        <v>42229.72325</v>
+        <v>15854.78</v>
       </c>
       <c r="M31" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N31" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -2184,16 +2223,16 @@
         <v>64</v>
       </c>
       <c r="G32" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L32">
-        <v>48857.39550000001</v>
+        <v>42229.72325</v>
       </c>
       <c r="M32" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N32" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="33" spans="1:16">
@@ -2204,54 +2243,36 @@
         <v>65</v>
       </c>
       <c r="G33" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L33">
-        <v>4192.68</v>
+        <v>48857.39550000001</v>
       </c>
       <c r="M33" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N33" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="34" spans="1:16">
       <c r="A34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B34" t="s">
         <v>66</v>
       </c>
-      <c r="D34">
-        <v>1465</v>
-      </c>
-      <c r="E34" s="2">
-        <v>46104</v>
-      </c>
-      <c r="F34" t="s">
-        <v>82</v>
-      </c>
-      <c r="H34" s="2">
-        <v>46106</v>
-      </c>
-      <c r="I34">
-        <v>27801.11</v>
-      </c>
-      <c r="J34" t="s">
-        <v>122</v>
-      </c>
-      <c r="K34">
-        <v>27801.11</v>
+      <c r="G34" t="s">
+        <v>97</v>
+      </c>
+      <c r="L34">
+        <v>4192.68</v>
       </c>
       <c r="M34" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="N34" t="s">
-        <v>126</v>
-      </c>
-      <c r="P34">
-        <v>1500000</v>
+        <v>131</v>
       </c>
     </row>
     <row r="35" spans="1:16">
@@ -2262,36 +2283,74 @@
         <v>67</v>
       </c>
       <c r="D35">
+        <v>1465</v>
+      </c>
+      <c r="E35" s="2">
+        <v>46104</v>
+      </c>
+      <c r="F35" t="s">
+        <v>83</v>
+      </c>
+      <c r="H35" s="2">
+        <v>46106</v>
+      </c>
+      <c r="I35">
+        <v>27801.11</v>
+      </c>
+      <c r="J35" t="s">
+        <v>126</v>
+      </c>
+      <c r="K35">
+        <v>27801.11</v>
+      </c>
+      <c r="M35" t="s">
+        <v>129</v>
+      </c>
+      <c r="N35" t="s">
+        <v>130</v>
+      </c>
+      <c r="P35">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16">
+      <c r="A36">
+        <v>3</v>
+      </c>
+      <c r="B36" t="s">
+        <v>68</v>
+      </c>
+      <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E36" s="2">
         <v>46199</v>
       </c>
-      <c r="F35" t="s">
-        <v>94</v>
-      </c>
-      <c r="H35" s="2">
+      <c r="F36" t="s">
+        <v>96</v>
+      </c>
+      <c r="H36" s="2">
         <v>46233</v>
       </c>
-      <c r="I35">
+      <c r="I36">
         <v>58868.35</v>
       </c>
-      <c r="J35" t="s">
-        <v>123</v>
-      </c>
-      <c r="K35">
+      <c r="J36" t="s">
+        <v>127</v>
+      </c>
+      <c r="K36">
         <v>58868.35</v>
       </c>
-      <c r="M35" t="s">
-        <v>125</v>
-      </c>
-      <c r="N35" t="s">
-        <v>127</v>
-      </c>
-      <c r="O35">
+      <c r="M36" t="s">
+        <v>129</v>
+      </c>
+      <c r="N36" t="s">
+        <v>132</v>
+      </c>
+      <c r="O36">
         <v>0.01</v>
       </c>
-      <c r="P35">
+      <c r="P36">
         <v>2364771.06</v>
       </c>
     </row>
@@ -2307,24 +2366,24 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B2">
         <v>1000</v>
@@ -2335,7 +2394,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B3">
         <v>52250.04</v>
@@ -2346,7 +2405,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B4">
         <v>881914.1800000001</v>
@@ -2357,7 +2416,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B5">
         <v>750000</v>
@@ -2368,7 +2427,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B6">
         <v>949835.78</v>
@@ -2379,7 +2438,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B7">
         <v>524584.95</v>
@@ -2390,7 +2449,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B8">
         <v>211614.23</v>
@@ -2401,7 +2460,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B9">
         <v>2391157.41</v>
@@ -2412,7 +2471,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B10">
         <v>618154.38</v>
@@ -2423,7 +2482,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B11">
         <v>1600334.09</v>
@@ -2434,7 +2493,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B12">
         <v>2364771.06</v>
@@ -2445,7 +2504,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B13">
         <v>968237.39</v>
@@ -2456,7 +2515,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B14">
         <v>1011677.95</v>
@@ -2467,7 +2526,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B15">
         <v>1580293.02</v>
@@ -2478,7 +2537,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B16">
         <v>0.01</v>
@@ -2489,7 +2548,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B17">
         <v>63746.85</v>
@@ -2500,7 +2559,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B18">
         <v>947931.1</v>
@@ -2511,7 +2570,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B19">
         <v>259790.57</v>
@@ -2522,7 +2581,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B20">
         <v>170479.3</v>
@@ -2533,7 +2592,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B21">
         <v>1500000</v>
@@ -2544,7 +2603,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B22">
         <v>1000001.64</v>
@@ -2555,7 +2614,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B23">
         <v>68405.66</v>
@@ -2566,7 +2625,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B24">
         <v>1157673.06</v>
@@ -2577,7 +2636,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B25">
         <v>34065.36</v>
@@ -2588,7 +2647,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B26">
         <v>843261.89</v>
@@ -2599,7 +2658,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B27">
         <v>1629834.48</v>
@@ -2610,7 +2669,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -2621,7 +2680,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -2632,7 +2691,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -2643,7 +2702,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B31">
         <v>0</v>
@@ -2654,7 +2713,7 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B32">
         <v>0</v>
@@ -2665,7 +2724,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -2676,7 +2735,7 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B34">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (28/09/2026 15:35)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,16 +509,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -534,7 +526,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -542,30 +534,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -865,37 +839,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -945,58 +919,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1013,13 +987,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1054,13 +1028,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1095,13 +1069,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1136,13 +1110,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1177,13 +1151,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1221,13 +1195,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1262,13 +1236,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1303,13 +1277,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1341,13 +1315,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1382,13 +1356,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1423,13 +1397,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1464,13 +1438,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1502,13 +1476,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1543,13 +1517,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1584,13 +1558,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1625,13 +1599,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1666,13 +1640,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1707,13 +1681,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1748,13 +1722,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1789,13 +1763,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1830,13 +1804,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1871,13 +1845,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1915,13 +1889,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1959,13 +1933,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -2003,13 +1977,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2044,13 +2018,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2085,13 +2059,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2126,13 +2100,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2167,13 +2141,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2285,13 +2259,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2323,13 +2297,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>96</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2365,19 +2339,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>134</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>135</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>136</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (29/09/2026 19:54)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,8 +509,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -526,7 +534,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -534,12 +542,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -839,37 +865,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -919,58 +945,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -987,13 +1013,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1028,13 +1054,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1069,13 +1095,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1110,13 +1136,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1151,13 +1177,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1195,13 +1221,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1236,13 +1262,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1277,13 +1303,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1315,13 +1341,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1356,13 +1382,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1397,13 +1423,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1438,13 +1464,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1476,13 +1502,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1517,13 +1543,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1558,13 +1584,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1599,13 +1625,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1640,13 +1666,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1681,13 +1707,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1722,13 +1748,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1763,13 +1789,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1804,13 +1830,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1845,13 +1871,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1889,13 +1915,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1933,13 +1959,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -1977,13 +2003,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2018,13 +2044,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2059,13 +2085,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2100,13 +2126,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2141,13 +2167,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2259,13 +2285,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2297,13 +2323,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>96</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2339,19 +2365,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>136</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (30/09/2026 13:48)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,16 +509,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -534,7 +526,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -542,30 +534,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -865,37 +839,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -945,58 +919,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1013,13 +987,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1054,13 +1028,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1095,13 +1069,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1136,13 +1110,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1177,13 +1151,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1221,13 +1195,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1262,13 +1236,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1303,13 +1277,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1341,13 +1315,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1382,13 +1356,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1423,13 +1397,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1464,13 +1438,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1502,13 +1476,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1543,13 +1517,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1584,13 +1558,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1625,13 +1599,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1666,13 +1640,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1707,13 +1681,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1748,13 +1722,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1789,13 +1763,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1830,13 +1804,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1871,13 +1845,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1915,13 +1889,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1959,13 +1933,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -2003,13 +1977,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2044,13 +2018,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2085,13 +2059,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2126,13 +2100,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2167,13 +2141,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2285,13 +2259,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2323,13 +2297,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>96</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2365,19 +2339,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>134</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>135</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>136</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (02/10/2026 09:56)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,8 +509,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -526,7 +534,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -534,12 +542,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -839,37 +865,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -919,58 +945,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -987,13 +1013,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1028,13 +1054,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1069,13 +1095,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1110,13 +1136,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1151,13 +1177,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1195,13 +1221,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1236,13 +1262,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1277,13 +1303,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1315,13 +1341,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1356,13 +1382,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1397,13 +1423,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1438,13 +1464,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1476,13 +1502,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1517,13 +1543,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1558,13 +1584,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1599,13 +1625,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1640,13 +1666,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1681,13 +1707,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1722,13 +1748,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1763,13 +1789,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1804,13 +1830,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1845,13 +1871,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1889,13 +1915,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1933,13 +1959,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -1977,13 +2003,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2018,13 +2044,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2059,13 +2085,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2100,13 +2126,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2141,13 +2167,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2259,13 +2285,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2297,13 +2323,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>96</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2339,19 +2365,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>136</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (02/10/2026 13:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,16 +509,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -534,7 +526,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -542,30 +534,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -865,37 +839,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -945,58 +919,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1013,13 +987,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1054,13 +1028,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1095,13 +1069,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1136,13 +1110,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1177,13 +1151,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1221,13 +1195,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1262,13 +1236,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1303,13 +1277,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1341,13 +1315,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1382,13 +1356,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1423,13 +1397,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1464,13 +1438,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1502,13 +1476,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1543,13 +1517,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1584,13 +1558,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1625,13 +1599,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1666,13 +1640,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1707,13 +1681,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1748,13 +1722,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1789,13 +1763,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1830,13 +1804,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1871,13 +1845,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1915,13 +1889,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1959,13 +1933,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -2003,13 +1977,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2044,13 +2018,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2085,13 +2059,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2126,13 +2100,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2167,13 +2141,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2285,13 +2259,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2323,13 +2297,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>96</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2365,19 +2339,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>134</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>135</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>136</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (05/10/2026 08:40)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,8 +509,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -526,7 +534,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -534,12 +542,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -839,37 +865,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -919,58 +945,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -987,13 +1013,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1028,13 +1054,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1069,13 +1095,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1110,13 +1136,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1151,13 +1177,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1195,13 +1221,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1236,13 +1262,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1277,13 +1303,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1315,13 +1341,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1356,13 +1382,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1397,13 +1423,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1438,13 +1464,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1476,13 +1502,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1517,13 +1543,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1558,13 +1584,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1599,13 +1625,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1640,13 +1666,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1681,13 +1707,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1722,13 +1748,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1763,13 +1789,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1804,13 +1830,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1845,13 +1871,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1889,13 +1915,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1933,13 +1959,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -1977,13 +2003,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2018,13 +2044,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2059,13 +2085,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2100,13 +2126,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2141,13 +2167,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2259,13 +2285,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2297,13 +2323,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>96</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2339,19 +2365,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>136</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (05/10/2026 15:52)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="160">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -310,10 +310,13 @@
     <t>2025NE001828</t>
   </si>
   <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
     <t>2025NE001065</t>
   </si>
   <si>
-    <t>Aprovado e aguardando itens</t>
+    <t>AGUARDANDO ITENS</t>
   </si>
   <si>
     <t>2025NP001980</t>
@@ -400,12 +403,12 @@
     <t>2026NP400445</t>
   </si>
   <si>
+    <t>Faturado</t>
+  </si>
+  <si>
     <t>2026NP401058</t>
   </si>
   <si>
-    <t>Faturado</t>
-  </si>
-  <si>
     <t>mensal</t>
   </si>
   <si>
@@ -415,12 +418,12 @@
     <t>Pago</t>
   </si>
   <si>
+    <t>Faturado, aguardando pagamento</t>
+  </si>
+  <si>
     <t>Pendente</t>
   </si>
   <si>
-    <t>Faturado, aguardando pagamento</t>
-  </si>
-  <si>
     <t>numero_empenho</t>
   </si>
   <si>
@@ -478,9 +481,6 @@
     <t>2025NE002237</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
     <t>2026NE000748</t>
   </si>
   <si>
@@ -499,7 +499,7 @@
     <t>2026NE001015</t>
   </si>
   <si>
-    <t>2026NE901182</t>
+    <t>2026NE001237</t>
   </si>
 </sst>
 </file>
@@ -1026,16 +1026,16 @@
         <v>748504.24</v>
       </c>
       <c r="J2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K2">
         <v>748504.24</v>
       </c>
       <c r="M2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P2">
         <v>881914.1800000001</v>
@@ -1067,16 +1067,16 @@
         <v>1110378.24</v>
       </c>
       <c r="J3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K3">
         <v>1110378.24</v>
       </c>
       <c r="M3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P3">
         <v>2634000</v>
@@ -1108,16 +1108,16 @@
         <v>974557.12</v>
       </c>
       <c r="J4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K4">
         <v>974557.12</v>
       </c>
       <c r="M4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P4">
         <v>1686034.96</v>
@@ -1149,16 +1149,16 @@
         <v>1402001.34</v>
       </c>
       <c r="J5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K5">
         <v>1402001.34</v>
       </c>
       <c r="M5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P5">
         <v>1600334.09</v>
@@ -1190,16 +1190,16 @@
         <v>1223702.3</v>
       </c>
       <c r="J6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K6">
         <v>1223702.3</v>
       </c>
       <c r="M6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O6">
         <v>0.02</v>
@@ -1234,16 +1234,16 @@
         <v>1011677.95</v>
       </c>
       <c r="J7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K7">
         <v>1011677.95</v>
       </c>
       <c r="M7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P7">
         <v>2568571.48</v>
@@ -1275,16 +1275,16 @@
         <v>896744.0600000001</v>
       </c>
       <c r="J8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K8">
         <v>896744.0600000001</v>
       </c>
       <c r="M8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P8">
         <v>968237.39</v>
@@ -1316,16 +1316,16 @@
         <v>919329.0600000001</v>
       </c>
       <c r="J9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K9">
         <v>919329.0600000001</v>
       </c>
       <c r="M9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P9">
         <v>1947932.74</v>
@@ -1354,16 +1354,16 @@
         <v>1157009.26</v>
       </c>
       <c r="J10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K10">
         <v>1157009.26</v>
       </c>
       <c r="M10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P10">
         <v>3105605.8</v>
@@ -1395,16 +1395,16 @@
         <v>1214597.952</v>
       </c>
       <c r="J11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K11">
         <v>1214597.952</v>
       </c>
       <c r="M11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P11">
         <v>2096487.74</v>
@@ -1436,16 +1436,16 @@
         <v>967082.09</v>
       </c>
       <c r="J12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K12">
         <v>967082.09</v>
       </c>
       <c r="M12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O12">
         <v>0.01</v>
@@ -1477,16 +1477,16 @@
         <v>719561.08</v>
       </c>
       <c r="J13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K13">
         <v>719561.08</v>
       </c>
       <c r="M13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P13">
         <v>1500000</v>
@@ -1515,16 +1515,16 @@
         <v>885881.08</v>
       </c>
       <c r="J14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K14">
         <v>885881.08</v>
       </c>
       <c r="M14" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N14" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O14">
         <v>34065.35</v>
@@ -1556,16 +1556,16 @@
         <v>1350542.52</v>
       </c>
       <c r="J15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K15">
         <v>1350542.52</v>
       </c>
       <c r="M15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O15">
         <v>0.01</v>
@@ -1597,16 +1597,16 @@
         <v>1108954.435833333</v>
       </c>
       <c r="J16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K16">
         <v>1108954.435833333</v>
       </c>
       <c r="M16" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O16">
         <v>0.02</v>
@@ -1638,16 +1638,16 @@
         <v>218206.1</v>
       </c>
       <c r="J17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K17">
         <v>218206.1</v>
       </c>
       <c r="M17" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N17" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O17">
         <v>0.02</v>
@@ -1679,16 +1679,16 @@
         <v>1549250.84</v>
       </c>
       <c r="J18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K18">
         <v>1549250.84</v>
       </c>
       <c r="M18" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N18" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O18">
         <v>0.02</v>
@@ -1720,22 +1720,22 @@
         <v>1340865.98</v>
       </c>
       <c r="J19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K19">
         <v>1340865.98</v>
       </c>
       <c r="M19" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N19" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O19">
-        <v>927618.62</v>
+        <v>306142.73</v>
       </c>
       <c r="P19">
-        <v>3208032.95</v>
+        <v>3829508.84</v>
       </c>
     </row>
     <row r="20" spans="1:16">
@@ -1761,22 +1761,19 @@
         <v>1629834.48</v>
       </c>
       <c r="J20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K20">
         <v>1629834.48</v>
       </c>
       <c r="M20" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N20" t="s">
-        <v>130</v>
-      </c>
-      <c r="O20">
-        <v>282458.04</v>
+        <v>131</v>
       </c>
       <c r="P20">
-        <v>1629834.48</v>
+        <v>1912292.52</v>
       </c>
     </row>
     <row r="21" spans="1:16">
@@ -1802,22 +1799,22 @@
         <v>1675964.21</v>
       </c>
       <c r="J21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K21">
         <v>1675964.21</v>
       </c>
       <c r="M21" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N21" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O21">
-        <v>2089048.83</v>
+        <v>306142.72</v>
       </c>
       <c r="P21">
-        <v>2473096.37</v>
+        <v>4256002.48</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -1843,16 +1840,16 @@
         <v>188246.17</v>
       </c>
       <c r="J22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K22">
         <v>188246.17</v>
       </c>
       <c r="M22" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P22">
         <v>211614.23</v>
@@ -1884,16 +1881,16 @@
         <v>112720.77</v>
       </c>
       <c r="J23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K23">
         <v>112720.77</v>
       </c>
       <c r="M23" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N23" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O23">
         <v>0.01</v>
@@ -1928,16 +1925,16 @@
         <v>378307.61</v>
       </c>
       <c r="J24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K24">
         <v>378307.61</v>
       </c>
       <c r="M24" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N24" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O24">
         <v>0.01</v>
@@ -1972,16 +1969,16 @@
         <v>3315.047100000025</v>
       </c>
       <c r="J25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K25">
         <v>3315.04710000003</v>
       </c>
       <c r="M25" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N25" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O25">
         <v>0.01</v>
@@ -2016,16 +2013,16 @@
         <v>198332.75</v>
       </c>
       <c r="J26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K26">
         <v>198332.75</v>
       </c>
       <c r="M26" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N26" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P26">
         <v>1600334.09</v>
@@ -2057,16 +2054,16 @@
         <v>1528.62</v>
       </c>
       <c r="J27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K27">
         <v>1528.62</v>
       </c>
       <c r="M27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N27" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P27">
         <v>1157673.06</v>
@@ -2098,16 +2095,16 @@
         <v>38718.58</v>
       </c>
       <c r="J28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K28">
         <v>38718.58</v>
       </c>
       <c r="M28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P28">
         <v>63746.85</v>
@@ -2139,16 +2136,16 @@
         <v>133124.11</v>
       </c>
       <c r="J29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K29">
         <v>133124.11</v>
       </c>
       <c r="M29" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P29">
         <v>1000001.64</v>
@@ -2180,16 +2177,16 @@
         <v>11372.9</v>
       </c>
       <c r="J30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K30">
         <v>11372.9</v>
       </c>
       <c r="M30" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N30" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P30">
         <v>1500000</v>
@@ -2202,17 +2199,38 @@
       <c r="B31" t="s">
         <v>63</v>
       </c>
-      <c r="G31" t="s">
-        <v>97</v>
-      </c>
-      <c r="L31">
+      <c r="D31">
+        <v>2243</v>
+      </c>
+      <c r="E31" s="2">
+        <v>46289</v>
+      </c>
+      <c r="F31" t="s">
+        <v>96</v>
+      </c>
+      <c r="H31" s="2">
+        <v>46325</v>
+      </c>
+      <c r="I31">
         <v>15854.78</v>
       </c>
+      <c r="J31" t="s">
+        <v>127</v>
+      </c>
+      <c r="K31">
+        <v>15854.78</v>
+      </c>
       <c r="M31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N31" t="s">
-        <v>131</v>
+        <v>132</v>
+      </c>
+      <c r="O31">
+        <v>306142.72</v>
+      </c>
+      <c r="P31">
+        <v>1464737.78</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -2222,17 +2240,35 @@
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="G32" t="s">
-        <v>97</v>
-      </c>
-      <c r="L32">
+      <c r="E32" s="2">
+        <v>46289</v>
+      </c>
+      <c r="F32" t="s">
+        <v>96</v>
+      </c>
+      <c r="H32" s="2">
+        <v>46325</v>
+      </c>
+      <c r="I32">
         <v>42229.72325</v>
       </c>
+      <c r="J32" t="s">
+        <v>127</v>
+      </c>
+      <c r="K32">
+        <v>42229.72325</v>
+      </c>
       <c r="M32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N32" t="s">
-        <v>131</v>
+        <v>132</v>
+      </c>
+      <c r="O32">
+        <v>306142.72</v>
+      </c>
+      <c r="P32">
+        <v>1464737.78</v>
       </c>
     </row>
     <row r="33" spans="1:16">
@@ -2242,17 +2278,35 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="G33" t="s">
-        <v>97</v>
-      </c>
-      <c r="L33">
+      <c r="E33" s="2">
+        <v>46289</v>
+      </c>
+      <c r="F33" t="s">
+        <v>96</v>
+      </c>
+      <c r="H33" s="2">
+        <v>46325</v>
+      </c>
+      <c r="I33">
         <v>48857.39550000001</v>
       </c>
+      <c r="J33" t="s">
+        <v>127</v>
+      </c>
+      <c r="K33">
+        <v>48857.39550000001</v>
+      </c>
       <c r="M33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N33" t="s">
-        <v>131</v>
+        <v>132</v>
+      </c>
+      <c r="O33">
+        <v>306142.72</v>
+      </c>
+      <c r="P33">
+        <v>1464737.78</v>
       </c>
     </row>
     <row r="34" spans="1:16">
@@ -2263,16 +2317,16 @@
         <v>66</v>
       </c>
       <c r="G34" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L34">
         <v>4192.68</v>
       </c>
       <c r="M34" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N34" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="35" spans="1:16">
@@ -2298,16 +2352,16 @@
         <v>27801.11</v>
       </c>
       <c r="J35" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="K35">
         <v>27801.11</v>
       </c>
       <c r="M35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P35">
         <v>1500000</v>
@@ -2327,7 +2381,7 @@
         <v>46199</v>
       </c>
       <c r="F36" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H36" s="2">
         <v>46233</v>
@@ -2342,7 +2396,7 @@
         <v>58868.35</v>
       </c>
       <c r="M36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N36" t="s">
         <v>132</v>
@@ -2366,24 +2420,24 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B2">
         <v>1000</v>
@@ -2394,7 +2448,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B3">
         <v>52250.04</v>
@@ -2405,7 +2459,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B4">
         <v>881914.1800000001</v>
@@ -2416,7 +2470,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B5">
         <v>750000</v>
@@ -2427,7 +2481,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B6">
         <v>949835.78</v>
@@ -2438,7 +2492,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B7">
         <v>524584.95</v>
@@ -2471,7 +2525,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B10">
         <v>618154.38</v>
@@ -2493,7 +2547,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B12">
         <v>2364771.06</v>
@@ -2515,7 +2569,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B14">
         <v>1011677.95</v>
@@ -2526,7 +2580,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B15">
         <v>1580293.02</v>
@@ -2537,7 +2591,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B16">
         <v>0.01</v>
@@ -2559,7 +2613,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B18">
         <v>947931.1</v>
@@ -2570,7 +2624,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B19">
         <v>259790.57</v>
@@ -2581,7 +2635,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B20">
         <v>170479.3</v>
@@ -2614,7 +2668,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B23">
         <v>68405.66</v>
@@ -2636,7 +2690,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B25">
         <v>34065.36</v>
@@ -2647,13 +2701,13 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>152</v>
+        <v>96</v>
       </c>
       <c r="B26">
-        <v>843261.89</v>
+        <v>1464737.78</v>
       </c>
       <c r="C26">
-        <v>927618.61</v>
+        <v>306142.72</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -2661,10 +2715,10 @@
         <v>88</v>
       </c>
       <c r="B27">
-        <v>1629834.48</v>
+        <v>1912292.52</v>
       </c>
       <c r="C27">
-        <v>282458.04</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -2683,10 +2737,10 @@
         <v>154</v>
       </c>
       <c r="B29">
+        <v>624166.14</v>
+      </c>
+      <c r="C29">
         <v>0</v>
-      </c>
-      <c r="C29">
-        <v>624166.14</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -2694,10 +2748,10 @@
         <v>155</v>
       </c>
       <c r="B30">
+        <v>18462.36</v>
+      </c>
+      <c r="C30">
         <v>0</v>
-      </c>
-      <c r="C30">
-        <v>18462.36</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -2727,10 +2781,10 @@
         <v>158</v>
       </c>
       <c r="B33">
+        <v>236343.68</v>
+      </c>
+      <c r="C33">
         <v>0</v>
-      </c>
-      <c r="C33">
-        <v>236343.68</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -2741,7 +2795,7 @@
         <v>0</v>
       </c>
       <c r="C34">
-        <v>1145462.93</v>
+        <v>1145462</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (06/10/2026 14:09)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,16 +509,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -534,7 +526,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -542,30 +534,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -865,37 +839,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -945,58 +919,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1013,13 +987,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1054,13 +1028,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1095,13 +1069,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1136,13 +1110,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1177,13 +1151,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1221,13 +1195,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1262,13 +1236,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1303,13 +1277,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1341,13 +1315,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1382,13 +1356,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1423,13 +1397,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1464,13 +1438,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1502,13 +1476,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1543,13 +1517,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1584,13 +1558,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1625,13 +1599,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1666,13 +1640,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1707,13 +1681,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1748,13 +1722,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1786,13 +1760,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1827,13 +1801,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1868,13 +1842,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1912,13 +1886,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1956,13 +1930,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -2000,13 +1974,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2041,13 +2015,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2082,13 +2056,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2123,13 +2097,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2164,13 +2138,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2202,13 +2176,13 @@
       <c r="D31">
         <v>2243</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46289</v>
       </c>
       <c r="F31" t="s">
         <v>96</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46325</v>
       </c>
       <c r="I31">
@@ -2240,13 +2214,13 @@
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>96</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2278,13 +2252,13 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>96</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2339,13 +2313,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2377,13 +2351,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>97</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2419,19 +2393,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>137</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (07/10/2026 11:10)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,8 +509,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -526,7 +534,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -534,12 +542,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -839,37 +865,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -919,58 +945,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -987,13 +1013,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1028,13 +1054,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1069,13 +1095,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1110,13 +1136,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1151,13 +1177,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1195,13 +1221,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1236,13 +1262,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1277,13 +1303,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1315,13 +1341,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1356,13 +1382,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1397,13 +1423,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1438,13 +1464,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1476,13 +1502,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1517,13 +1543,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1558,13 +1584,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1599,13 +1625,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1640,13 +1666,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1681,13 +1707,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1722,13 +1748,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1760,13 +1786,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1801,13 +1827,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1842,13 +1868,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1886,13 +1912,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1930,13 +1956,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -1974,13 +2000,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2015,13 +2041,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2056,13 +2082,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2097,13 +2123,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2138,13 +2164,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2176,13 +2202,13 @@
       <c r="D31">
         <v>2243</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46289</v>
       </c>
       <c r="F31" t="s">
         <v>96</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46325</v>
       </c>
       <c r="I31">
@@ -2214,13 +2240,13 @@
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>96</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2252,13 +2278,13 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>96</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2313,13 +2339,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2351,13 +2377,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>97</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2393,19 +2419,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>137</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (07/10/2026 14:46)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,16 +509,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -534,7 +526,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -542,30 +534,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -865,37 +839,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -945,58 +919,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1013,13 +987,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1054,13 +1028,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1095,13 +1069,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1136,13 +1110,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1177,13 +1151,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1221,13 +1195,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1262,13 +1236,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1303,13 +1277,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1341,13 +1315,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1382,13 +1356,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1423,13 +1397,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1464,13 +1438,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1502,13 +1476,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1543,13 +1517,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1584,13 +1558,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1625,13 +1599,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1666,13 +1640,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1707,13 +1681,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1748,13 +1722,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1786,13 +1760,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1827,13 +1801,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1868,13 +1842,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1912,13 +1886,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1956,13 +1930,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -2000,13 +1974,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2041,13 +2015,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2082,13 +2056,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2123,13 +2097,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2164,13 +2138,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2202,13 +2176,13 @@
       <c r="D31">
         <v>2243</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46289</v>
       </c>
       <c r="F31" t="s">
         <v>96</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46325</v>
       </c>
       <c r="I31">
@@ -2240,13 +2214,13 @@
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>96</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2278,13 +2252,13 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>96</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2339,13 +2313,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2377,13 +2351,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>97</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2419,19 +2393,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>137</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (13/10/2026 10:13)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,8 +509,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -526,7 +534,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -534,12 +542,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -839,37 +865,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -919,58 +945,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -987,13 +1013,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1028,13 +1054,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1069,13 +1095,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1110,13 +1136,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1151,13 +1177,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1195,13 +1221,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1236,13 +1262,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1277,13 +1303,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1315,13 +1341,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1356,13 +1382,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1397,13 +1423,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1438,13 +1464,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1476,13 +1502,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1517,13 +1543,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1558,13 +1584,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1599,13 +1625,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1640,13 +1666,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1681,13 +1707,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1722,13 +1748,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1760,13 +1786,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1801,13 +1827,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1842,13 +1868,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1886,13 +1912,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1930,13 +1956,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -1974,13 +2000,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2015,13 +2041,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2056,13 +2082,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2097,13 +2123,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2138,13 +2164,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2176,13 +2202,13 @@
       <c r="D31">
         <v>2243</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46289</v>
       </c>
       <c r="F31" t="s">
         <v>96</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46325</v>
       </c>
       <c r="I31">
@@ -2214,13 +2240,13 @@
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>96</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2252,13 +2278,13 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>96</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2313,13 +2339,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2351,13 +2377,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>97</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2393,19 +2419,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>137</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (13/10/2026 15:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,16 +509,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -534,7 +526,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -542,30 +534,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -865,37 +839,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -945,58 +919,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1013,13 +987,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1054,13 +1028,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1095,13 +1069,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1136,13 +1110,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1177,13 +1151,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1221,13 +1195,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1262,13 +1236,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1303,13 +1277,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1341,13 +1315,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1382,13 +1356,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1423,13 +1397,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1464,13 +1438,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1502,13 +1476,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1543,13 +1517,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1584,13 +1558,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1625,13 +1599,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1666,13 +1640,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1707,13 +1681,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1748,13 +1722,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1786,13 +1760,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1827,13 +1801,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1868,13 +1842,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1912,13 +1886,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1956,13 +1930,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -2000,13 +1974,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2041,13 +2015,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2082,13 +2056,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2123,13 +2097,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2164,13 +2138,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2202,13 +2176,13 @@
       <c r="D31">
         <v>2243</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46289</v>
       </c>
       <c r="F31" t="s">
         <v>96</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46325</v>
       </c>
       <c r="I31">
@@ -2240,13 +2214,13 @@
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>96</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2278,13 +2252,13 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>96</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2339,13 +2313,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2377,13 +2351,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>97</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2419,19 +2393,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>137</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (14/10/2026 13:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -509,8 +509,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -526,7 +534,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -534,12 +542,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -839,37 +865,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -919,58 +945,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -987,13 +1013,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1028,13 +1054,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1069,13 +1095,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1110,13 +1136,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1151,13 +1177,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1195,13 +1221,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1236,13 +1262,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1277,13 +1303,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1315,13 +1341,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1356,13 +1382,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1397,13 +1423,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1438,13 +1464,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1476,13 +1502,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1517,13 +1543,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1558,13 +1584,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1599,13 +1625,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1640,13 +1666,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1681,13 +1707,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1722,13 +1748,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1760,13 +1786,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1801,13 +1827,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1842,13 +1868,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1886,13 +1912,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1930,13 +1956,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -1974,13 +2000,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2015,13 +2041,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2056,13 +2082,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2097,13 +2123,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2138,13 +2164,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2176,13 +2202,13 @@
       <c r="D31">
         <v>2243</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46289</v>
       </c>
       <c r="F31" t="s">
         <v>96</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46325</v>
       </c>
       <c r="I31">
@@ -2214,13 +2240,13 @@
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>96</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2252,13 +2278,13 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>96</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2313,13 +2339,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2351,13 +2377,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>97</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2393,19 +2419,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>137</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (15/10/2026 12:34)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="166">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -500,6 +500,24 @@
   </si>
   <si>
     <t>2026NE001237</t>
+  </si>
+  <si>
+    <t>2026NE001294</t>
+  </si>
+  <si>
+    <t>2026NE001360</t>
+  </si>
+  <si>
+    <t>2026NE001383</t>
+  </si>
+  <si>
+    <t>2026NE001384</t>
+  </si>
+  <si>
+    <t>2026NE001457</t>
+  </si>
+  <si>
+    <t>2026NE001551</t>
   </si>
 </sst>
 </file>
@@ -509,16 +527,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -534,7 +544,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -542,30 +552,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -865,37 +857,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -945,58 +937,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1013,13 +1005,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1054,13 +1046,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1095,13 +1087,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1136,13 +1128,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1177,13 +1169,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1221,13 +1213,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1262,13 +1254,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1303,13 +1295,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1341,13 +1333,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1382,13 +1374,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1423,13 +1415,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1464,13 +1456,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1502,13 +1494,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1527,10 +1519,10 @@
         <v>131</v>
       </c>
       <c r="O14">
-        <v>34065.35</v>
+        <v>34065.36</v>
       </c>
       <c r="P14">
-        <v>3080293.03</v>
+        <v>3080293.02</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -1543,13 +1535,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1584,13 +1576,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1625,13 +1617,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1666,13 +1658,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1707,13 +1699,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1732,10 +1724,10 @@
         <v>131</v>
       </c>
       <c r="O19">
-        <v>306142.73</v>
+        <v>306142.72</v>
       </c>
       <c r="P19">
-        <v>3829508.84</v>
+        <v>3829508.85</v>
       </c>
     </row>
     <row r="20" spans="1:16">
@@ -1748,13 +1740,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1786,13 +1778,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1811,10 +1803,10 @@
         <v>131</v>
       </c>
       <c r="O21">
-        <v>306142.72</v>
+        <v>306142.71</v>
       </c>
       <c r="P21">
-        <v>4256002.48</v>
+        <v>4256002.49</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -1827,13 +1819,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1868,13 +1860,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1912,13 +1904,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1956,13 +1948,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -2000,13 +1992,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2041,13 +2033,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2082,13 +2074,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2123,13 +2115,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2164,13 +2156,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2202,13 +2194,13 @@
       <c r="D31">
         <v>2243</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46289</v>
       </c>
       <c r="F31" t="s">
         <v>96</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46325</v>
       </c>
       <c r="I31">
@@ -2227,10 +2219,10 @@
         <v>132</v>
       </c>
       <c r="O31">
-        <v>306142.72</v>
+        <v>306142.71</v>
       </c>
       <c r="P31">
-        <v>1464737.78</v>
+        <v>1464737.79</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -2240,13 +2232,13 @@
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>96</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2265,10 +2257,10 @@
         <v>132</v>
       </c>
       <c r="O32">
-        <v>306142.72</v>
+        <v>306142.71</v>
       </c>
       <c r="P32">
-        <v>1464737.78</v>
+        <v>1464737.79</v>
       </c>
     </row>
     <row r="33" spans="1:16">
@@ -2278,13 +2270,13 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>96</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2303,10 +2295,10 @@
         <v>132</v>
       </c>
       <c r="O33">
-        <v>306142.72</v>
+        <v>306142.71</v>
       </c>
       <c r="P33">
-        <v>1464737.78</v>
+        <v>1464737.79</v>
       </c>
     </row>
     <row r="34" spans="1:16">
@@ -2339,13 +2331,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="1">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="1">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2377,13 +2369,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>97</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2415,23 +2407,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>137</v>
       </c>
     </row>
@@ -2594,10 +2586,10 @@
         <v>147</v>
       </c>
       <c r="B16">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="C16">
-        <v>34065.35</v>
+        <v>34065.36</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -2704,10 +2696,10 @@
         <v>96</v>
       </c>
       <c r="B26">
-        <v>1464737.78</v>
+        <v>1464737.79</v>
       </c>
       <c r="C26">
-        <v>306142.72</v>
+        <v>306142.71</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -2795,7 +2787,73 @@
         <v>0</v>
       </c>
       <c r="C34">
-        <v>1145462</v>
+        <v>1145462.93</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>160</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35">
+        <v>859536.0699999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>161</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36">
+        <v>389619.06</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>162</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37">
+        <v>66366.75999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>163</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>103054.25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>164</v>
+      </c>
+      <c r="B39">
+        <v>0</v>
+      </c>
+      <c r="C39">
+        <v>1295422.28</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>165</v>
+      </c>
+      <c r="B40">
+        <v>0</v>
+      </c>
+      <c r="C40">
+        <v>117742.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (16/10/2026 12:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -527,8 +527,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -544,7 +552,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -552,12 +560,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -857,37 +883,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -937,58 +963,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1005,13 +1031,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1046,13 +1072,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1087,13 +1113,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1128,13 +1154,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1169,13 +1195,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>76</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1213,13 +1239,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>77</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1254,13 +1280,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1295,13 +1321,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1333,13 +1359,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1374,13 +1400,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1415,13 +1441,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1456,13 +1482,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1494,13 +1520,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1535,13 +1561,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1576,13 +1602,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1617,13 +1643,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1658,13 +1684,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1699,13 +1725,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1740,13 +1766,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1778,13 +1804,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1819,13 +1845,13 @@
       <c r="D22">
         <v>402</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45791</v>
       </c>
       <c r="F22" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45834</v>
       </c>
       <c r="I22">
@@ -1860,13 +1886,13 @@
       <c r="D23">
         <v>447</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45814</v>
       </c>
       <c r="F23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45955</v>
       </c>
       <c r="I23">
@@ -1904,13 +1930,13 @@
       <c r="D24">
         <v>529</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45853</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45939</v>
       </c>
       <c r="I24">
@@ -1948,13 +1974,13 @@
       <c r="D25">
         <v>691</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45910</v>
       </c>
       <c r="F25" t="s">
         <v>92</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45941</v>
       </c>
       <c r="I25">
@@ -1992,13 +2018,13 @@
       <c r="D26">
         <v>677</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45904</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2033,13 +2059,13 @@
       <c r="D27">
         <v>278</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>46008</v>
       </c>
       <c r="F27" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>46066</v>
       </c>
       <c r="I27">
@@ -2074,13 +2100,13 @@
       <c r="D28">
         <v>748</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45930</v>
       </c>
       <c r="F28" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2115,13 +2141,13 @@
       <c r="D29">
         <v>822</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45968</v>
       </c>
       <c r="F29" t="s">
         <v>95</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2156,13 +2182,13 @@
       <c r="D30">
         <v>360</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>46043</v>
       </c>
       <c r="F30" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46075</v>
       </c>
       <c r="I30">
@@ -2194,13 +2220,13 @@
       <c r="D31">
         <v>2243</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46289</v>
       </c>
       <c r="F31" t="s">
         <v>96</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46325</v>
       </c>
       <c r="I31">
@@ -2232,13 +2258,13 @@
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>96</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2270,13 +2296,13 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>96</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2331,13 +2357,13 @@
       <c r="D35">
         <v>1465</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="2">
         <v>46104</v>
       </c>
       <c r="F35" t="s">
         <v>83</v>
       </c>
-      <c r="H35" s="1">
+      <c r="H35" s="2">
         <v>46106</v>
       </c>
       <c r="I35">
@@ -2369,13 +2395,13 @@
       <c r="D36">
         <v>1882</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46199</v>
       </c>
       <c r="F36" t="s">
         <v>97</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46233</v>
       </c>
       <c r="I36">
@@ -2411,19 +2437,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>137</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (16/10/2026 12:21)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="168">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -178,6 +178,9 @@
   </si>
   <si>
     <t>AGOSTO/26</t>
+  </si>
+  <si>
+    <t>SETEMBRO/26</t>
   </si>
   <si>
     <t>Módulo II – Parcial Orçamento 10 (FAB 2728)</t>
@@ -290,6 +293,9 @@
   </si>
   <si>
     <t>2026NE000330, 2026NE000388, 2026NE000816, 2026NE000817, 2026NE001015</t>
+  </si>
+  <si>
+    <t>2026NE001551, 2026NE000842</t>
   </si>
   <si>
     <t>2025NE000559</t>
@@ -527,16 +533,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -552,7 +550,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -560,30 +558,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -883,37 +863,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -959,62 +939,62 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R36"/>
+  <dimension ref="A1:R37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1026,34 +1006,34 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H2" s="2">
+        <v>73</v>
+      </c>
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
         <v>748504.24</v>
       </c>
       <c r="J2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K2">
         <v>748504.24</v>
       </c>
       <c r="M2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P2">
         <v>881914.1800000001</v>
@@ -1067,34 +1047,34 @@
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
-        <v>73</v>
-      </c>
-      <c r="H3" s="2">
+        <v>74</v>
+      </c>
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
         <v>1110378.24</v>
       </c>
       <c r="J3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K3">
         <v>1110378.24</v>
       </c>
       <c r="M3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P3">
         <v>2634000</v>
@@ -1108,34 +1088,34 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
-        <v>74</v>
-      </c>
-      <c r="H4" s="2">
+        <v>75</v>
+      </c>
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
         <v>974557.12</v>
       </c>
       <c r="J4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="K4">
         <v>974557.12</v>
       </c>
       <c r="M4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P4">
         <v>1686034.96</v>
@@ -1149,34 +1129,34 @@
         <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
-      </c>
-      <c r="H5" s="2">
+        <v>76</v>
+      </c>
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
         <v>1402001.34</v>
       </c>
       <c r="J5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K5">
         <v>1402001.34</v>
       </c>
       <c r="M5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P5">
         <v>1600334.09</v>
@@ -1190,34 +1170,34 @@
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
-      </c>
-      <c r="H6" s="2">
+        <v>77</v>
+      </c>
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
         <v>1223702.3</v>
       </c>
       <c r="J6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="K6">
         <v>1223702.3</v>
       </c>
       <c r="M6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O6">
         <v>0.02</v>
@@ -1234,34 +1214,34 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
-      </c>
-      <c r="H7" s="2">
+        <v>78</v>
+      </c>
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
         <v>1011677.95</v>
       </c>
       <c r="J7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K7">
         <v>1011677.95</v>
       </c>
       <c r="M7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N7" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P7">
         <v>2568571.48</v>
@@ -1275,34 +1255,34 @@
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
-        <v>78</v>
-      </c>
-      <c r="H8" s="2">
+        <v>79</v>
+      </c>
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
         <v>896744.0600000001</v>
       </c>
       <c r="J8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="K8">
         <v>896744.0600000001</v>
       </c>
       <c r="M8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P8">
         <v>968237.39</v>
@@ -1316,34 +1296,34 @@
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
-        <v>79</v>
-      </c>
-      <c r="H9" s="2">
+        <v>80</v>
+      </c>
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
         <v>919329.0600000001</v>
       </c>
       <c r="J9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K9">
         <v>919329.0600000001</v>
       </c>
       <c r="M9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P9">
         <v>1947932.74</v>
@@ -1359,29 +1339,29 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
-        <v>80</v>
-      </c>
-      <c r="H10" s="2">
+        <v>81</v>
+      </c>
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
         <v>1157009.26</v>
       </c>
       <c r="J10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K10">
         <v>1157009.26</v>
       </c>
       <c r="M10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P10">
         <v>3105605.8</v>
@@ -1395,34 +1375,34 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
-        <v>81</v>
-      </c>
-      <c r="H11" s="2">
+        <v>82</v>
+      </c>
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
         <v>1214597.952</v>
       </c>
       <c r="J11" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K11">
         <v>1214597.952</v>
       </c>
       <c r="M11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P11">
         <v>2096487.74</v>
@@ -1436,34 +1416,34 @@
         <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
-        <v>82</v>
-      </c>
-      <c r="H12" s="2">
+        <v>83</v>
+      </c>
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
         <v>967082.09</v>
       </c>
       <c r="J12" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="K12">
         <v>967082.09</v>
       </c>
       <c r="M12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O12">
         <v>0.01</v>
@@ -1482,29 +1462,29 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
-        <v>83</v>
-      </c>
-      <c r="H13" s="2">
+        <v>84</v>
+      </c>
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
         <v>719561.08</v>
       </c>
       <c r="J13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K13">
         <v>719561.08</v>
       </c>
       <c r="M13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N13" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P13">
         <v>1500000</v>
@@ -1520,29 +1500,29 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
-        <v>84</v>
-      </c>
-      <c r="H14" s="2">
+        <v>85</v>
+      </c>
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
         <v>885881.08</v>
       </c>
       <c r="J14" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="K14">
         <v>885881.08</v>
       </c>
       <c r="M14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O14">
         <v>34065.36</v>
@@ -1561,29 +1541,29 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
-      </c>
-      <c r="H15" s="2">
+        <v>86</v>
+      </c>
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
         <v>1350542.52</v>
       </c>
       <c r="J15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K15">
         <v>1350542.52</v>
       </c>
       <c r="M15" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O15">
         <v>0.01</v>
@@ -1602,29 +1582,29 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
-        <v>86</v>
-      </c>
-      <c r="H16" s="2">
+        <v>87</v>
+      </c>
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
         <v>1108954.435833333</v>
       </c>
       <c r="J16" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="K16">
         <v>1108954.435833333</v>
       </c>
       <c r="M16" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N16" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O16">
         <v>0.02</v>
@@ -1643,29 +1623,29 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
-        <v>86</v>
-      </c>
-      <c r="H17" s="2">
+        <v>87</v>
+      </c>
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
         <v>218206.1</v>
       </c>
       <c r="J17" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K17">
         <v>218206.1</v>
       </c>
       <c r="M17" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N17" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O17">
         <v>0.02</v>
@@ -1684,29 +1664,29 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
-        <v>86</v>
-      </c>
-      <c r="H18" s="2">
+        <v>87</v>
+      </c>
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
         <v>1549250.84</v>
       </c>
       <c r="J18" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K18">
         <v>1549250.84</v>
       </c>
       <c r="M18" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N18" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O18">
         <v>0.02</v>
@@ -1725,29 +1705,29 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
-        <v>87</v>
-      </c>
-      <c r="H19" s="2">
+        <v>88</v>
+      </c>
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
         <v>1340865.98</v>
       </c>
       <c r="J19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="K19">
         <v>1340865.98</v>
       </c>
       <c r="M19" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N19" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O19">
         <v>306142.72</v>
@@ -1766,29 +1746,29 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
-        <v>88</v>
-      </c>
-      <c r="H20" s="2">
+        <v>89</v>
+      </c>
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="I20">
         <v>1629834.48</v>
       </c>
       <c r="J20" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K20">
         <v>1629834.48</v>
       </c>
       <c r="M20" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N20" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P20">
         <v>1912292.52</v>
@@ -1804,29 +1784,29 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
-        <v>89</v>
-      </c>
-      <c r="H21" s="2">
+        <v>90</v>
+      </c>
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
         <v>1675964.21</v>
       </c>
       <c r="J21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="K21">
         <v>1675964.21</v>
       </c>
       <c r="M21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N21" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O21">
         <v>306142.71</v>
@@ -1837,40 +1817,31 @@
     </row>
     <row r="22" spans="1:16">
       <c r="A22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B22" t="s">
         <v>54</v>
       </c>
       <c r="D22">
-        <v>402</v>
-      </c>
-      <c r="E22" s="2">
-        <v>45791</v>
+        <v>71</v>
+      </c>
+      <c r="E22" s="1">
+        <v>46309</v>
       </c>
       <c r="F22" t="s">
-        <v>90</v>
-      </c>
-      <c r="H22" s="2">
-        <v>45834</v>
+        <v>91</v>
       </c>
       <c r="I22">
-        <v>188246.17</v>
-      </c>
-      <c r="J22" t="s">
-        <v>118</v>
-      </c>
-      <c r="K22">
-        <v>188246.17</v>
+        <v>1565507.76</v>
       </c>
       <c r="M22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="N22" t="s">
-        <v>131</v>
-      </c>
-      <c r="P22">
-        <v>211614.23</v>
+        <v>134</v>
+      </c>
+      <c r="O22">
+        <v>1648399.2</v>
       </c>
     </row>
     <row r="23" spans="1:16">
@@ -1880,41 +1851,35 @@
       <c r="B23" t="s">
         <v>55</v>
       </c>
-      <c r="C23">
-        <v>46</v>
-      </c>
       <c r="D23">
-        <v>447</v>
-      </c>
-      <c r="E23" s="2">
-        <v>45814</v>
+        <v>402</v>
+      </c>
+      <c r="E23" s="1">
+        <v>45791</v>
       </c>
       <c r="F23" t="s">
-        <v>91</v>
-      </c>
-      <c r="H23" s="2">
-        <v>45955</v>
+        <v>92</v>
+      </c>
+      <c r="H23" s="1">
+        <v>45834</v>
       </c>
       <c r="I23">
-        <v>112720.77</v>
+        <v>188246.17</v>
       </c>
       <c r="J23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K23">
-        <v>112720.77</v>
+        <v>188246.17</v>
       </c>
       <c r="M23" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N23" t="s">
-        <v>131</v>
-      </c>
-      <c r="O23">
-        <v>0.01</v>
+        <v>133</v>
       </c>
       <c r="P23">
-        <v>3359394.8</v>
+        <v>211614.23</v>
       </c>
     </row>
     <row r="24" spans="1:16">
@@ -1924,41 +1889,41 @@
       <c r="B24" t="s">
         <v>56</v>
       </c>
-      <c r="C24" t="s">
-        <v>70</v>
+      <c r="C24">
+        <v>46</v>
       </c>
       <c r="D24">
-        <v>529</v>
-      </c>
-      <c r="E24" s="2">
-        <v>45853</v>
+        <v>447</v>
+      </c>
+      <c r="E24" s="1">
+        <v>45814</v>
       </c>
       <c r="F24" t="s">
-        <v>92</v>
-      </c>
-      <c r="H24" s="2">
-        <v>45939</v>
+        <v>93</v>
+      </c>
+      <c r="H24" s="1">
+        <v>45955</v>
       </c>
       <c r="I24">
-        <v>378307.61</v>
+        <v>112720.77</v>
       </c>
       <c r="J24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K24">
-        <v>378307.61</v>
+        <v>112720.77</v>
       </c>
       <c r="M24" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N24" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O24">
         <v>0.01</v>
       </c>
       <c r="P24">
-        <v>2391157.41</v>
+        <v>3359394.8</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -1969,34 +1934,34 @@
         <v>57</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D25">
-        <v>691</v>
-      </c>
-      <c r="E25" s="2">
-        <v>45910</v>
+        <v>529</v>
+      </c>
+      <c r="E25" s="1">
+        <v>45853</v>
       </c>
       <c r="F25" t="s">
-        <v>92</v>
-      </c>
-      <c r="H25" s="2">
-        <v>45941</v>
+        <v>94</v>
+      </c>
+      <c r="H25" s="1">
+        <v>45939</v>
       </c>
       <c r="I25">
-        <v>3315.047100000025</v>
+        <v>378307.61</v>
       </c>
       <c r="J25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K25">
-        <v>3315.04710000003</v>
+        <v>378307.61</v>
       </c>
       <c r="M25" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N25" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O25">
         <v>0.01</v>
@@ -2012,38 +1977,41 @@
       <c r="B26" t="s">
         <v>58</v>
       </c>
-      <c r="C26">
-        <v>135</v>
+      <c r="C26" t="s">
+        <v>71</v>
       </c>
       <c r="D26">
-        <v>677</v>
-      </c>
-      <c r="E26" s="2">
-        <v>45904</v>
+        <v>691</v>
+      </c>
+      <c r="E26" s="1">
+        <v>45910</v>
       </c>
       <c r="F26" t="s">
-        <v>75</v>
-      </c>
-      <c r="H26" s="2">
-        <v>45935</v>
+        <v>94</v>
+      </c>
+      <c r="H26" s="1">
+        <v>45941</v>
       </c>
       <c r="I26">
-        <v>198332.75</v>
+        <v>3315.047100000025</v>
       </c>
       <c r="J26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K26">
-        <v>198332.75</v>
+        <v>3315.04710000003</v>
       </c>
       <c r="M26" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N26" t="s">
-        <v>131</v>
+        <v>133</v>
+      </c>
+      <c r="O26">
+        <v>0.01</v>
       </c>
       <c r="P26">
-        <v>1600334.09</v>
+        <v>2391157.41</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -2054,37 +2022,37 @@
         <v>59</v>
       </c>
       <c r="C27">
-        <v>40</v>
+        <v>135</v>
       </c>
       <c r="D27">
-        <v>278</v>
-      </c>
-      <c r="E27" s="2">
-        <v>46008</v>
+        <v>677</v>
+      </c>
+      <c r="E27" s="1">
+        <v>45904</v>
       </c>
       <c r="F27" t="s">
-        <v>93</v>
-      </c>
-      <c r="H27" s="2">
-        <v>46066</v>
+        <v>76</v>
+      </c>
+      <c r="H27" s="1">
+        <v>45935</v>
       </c>
       <c r="I27">
-        <v>1528.62</v>
+        <v>198332.75</v>
       </c>
       <c r="J27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K27">
-        <v>1528.62</v>
+        <v>198332.75</v>
       </c>
       <c r="M27" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N27" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P27">
-        <v>1157673.06</v>
+        <v>1600334.09</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -2094,38 +2062,38 @@
       <c r="B28" t="s">
         <v>60</v>
       </c>
-      <c r="C28" t="s">
-        <v>71</v>
+      <c r="C28">
+        <v>40</v>
       </c>
       <c r="D28">
-        <v>748</v>
-      </c>
-      <c r="E28" s="2">
-        <v>45930</v>
+        <v>278</v>
+      </c>
+      <c r="E28" s="1">
+        <v>46008</v>
       </c>
       <c r="F28" t="s">
-        <v>94</v>
-      </c>
-      <c r="H28" s="2">
-        <v>45935</v>
+        <v>95</v>
+      </c>
+      <c r="H28" s="1">
+        <v>46066</v>
       </c>
       <c r="I28">
-        <v>38718.58</v>
+        <v>1528.62</v>
       </c>
       <c r="J28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K28">
-        <v>38718.58</v>
+        <v>1528.62</v>
       </c>
       <c r="M28" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N28" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P28">
-        <v>63746.85</v>
+        <v>1157673.06</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -2135,38 +2103,38 @@
       <c r="B29" t="s">
         <v>61</v>
       </c>
-      <c r="C29">
-        <v>154</v>
+      <c r="C29" t="s">
+        <v>72</v>
       </c>
       <c r="D29">
-        <v>822</v>
-      </c>
-      <c r="E29" s="2">
-        <v>45968</v>
+        <v>748</v>
+      </c>
+      <c r="E29" s="1">
+        <v>45930</v>
       </c>
       <c r="F29" t="s">
-        <v>95</v>
-      </c>
-      <c r="H29" s="2">
+        <v>96</v>
+      </c>
+      <c r="H29" s="1">
         <v>45935</v>
       </c>
       <c r="I29">
-        <v>133124.11</v>
+        <v>38718.58</v>
       </c>
       <c r="J29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K29">
-        <v>133124.11</v>
+        <v>38718.58</v>
       </c>
       <c r="M29" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N29" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P29">
-        <v>1000001.64</v>
+        <v>63746.85</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -2177,37 +2145,37 @@
         <v>62</v>
       </c>
       <c r="C30">
-        <v>252</v>
+        <v>154</v>
       </c>
       <c r="D30">
-        <v>360</v>
-      </c>
-      <c r="E30" s="2">
-        <v>46043</v>
+        <v>822</v>
+      </c>
+      <c r="E30" s="1">
+        <v>45968</v>
       </c>
       <c r="F30" t="s">
-        <v>83</v>
-      </c>
-      <c r="H30" s="2">
-        <v>46075</v>
+        <v>97</v>
+      </c>
+      <c r="H30" s="1">
+        <v>45935</v>
       </c>
       <c r="I30">
-        <v>11372.9</v>
+        <v>133124.11</v>
       </c>
       <c r="J30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K30">
-        <v>11372.9</v>
+        <v>133124.11</v>
       </c>
       <c r="M30" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N30" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="P30">
-        <v>1500000</v>
+        <v>1000001.64</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -2217,38 +2185,38 @@
       <c r="B31" t="s">
         <v>63</v>
       </c>
+      <c r="C31">
+        <v>252</v>
+      </c>
       <c r="D31">
-        <v>2243</v>
-      </c>
-      <c r="E31" s="2">
-        <v>46289</v>
+        <v>360</v>
+      </c>
+      <c r="E31" s="1">
+        <v>46043</v>
       </c>
       <c r="F31" t="s">
-        <v>96</v>
-      </c>
-      <c r="H31" s="2">
-        <v>46325</v>
+        <v>84</v>
+      </c>
+      <c r="H31" s="1">
+        <v>46075</v>
       </c>
       <c r="I31">
-        <v>15854.78</v>
+        <v>11372.9</v>
       </c>
       <c r="J31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K31">
-        <v>15854.78</v>
+        <v>11372.9</v>
       </c>
       <c r="M31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N31" t="s">
-        <v>132</v>
-      </c>
-      <c r="O31">
-        <v>306142.71</v>
+        <v>133</v>
       </c>
       <c r="P31">
-        <v>1464737.79</v>
+        <v>1500000</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -2258,29 +2226,32 @@
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="E32" s="2">
+      <c r="D32">
+        <v>2243</v>
+      </c>
+      <c r="E32" s="1">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
-        <v>96</v>
-      </c>
-      <c r="H32" s="2">
+        <v>98</v>
+      </c>
+      <c r="H32" s="1">
         <v>46325</v>
       </c>
       <c r="I32">
-        <v>42229.72325</v>
+        <v>15854.78</v>
       </c>
       <c r="J32" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K32">
-        <v>42229.72325</v>
+        <v>15854.78</v>
       </c>
       <c r="M32" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N32" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="O32">
         <v>306142.71</v>
@@ -2296,29 +2267,29 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
-        <v>96</v>
-      </c>
-      <c r="H33" s="2">
+        <v>98</v>
+      </c>
+      <c r="H33" s="1">
         <v>46325</v>
       </c>
       <c r="I33">
-        <v>48857.39550000001</v>
+        <v>42229.72325</v>
       </c>
       <c r="J33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K33">
-        <v>48857.39550000001</v>
+        <v>42229.72325</v>
       </c>
       <c r="M33" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="O33">
         <v>306142.71</v>
@@ -2334,55 +2305,55 @@
       <c r="B34" t="s">
         <v>66</v>
       </c>
-      <c r="G34" t="s">
+      <c r="E34" s="1">
+        <v>46289</v>
+      </c>
+      <c r="F34" t="s">
         <v>98</v>
       </c>
-      <c r="L34">
-        <v>4192.68</v>
+      <c r="H34" s="1">
+        <v>46325</v>
+      </c>
+      <c r="I34">
+        <v>48857.39550000001</v>
+      </c>
+      <c r="J34" t="s">
+        <v>129</v>
+      </c>
+      <c r="K34">
+        <v>48857.39550000001</v>
       </c>
       <c r="M34" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N34" t="s">
-        <v>133</v>
+        <v>134</v>
+      </c>
+      <c r="O34">
+        <v>306142.71</v>
+      </c>
+      <c r="P34">
+        <v>1464737.79</v>
       </c>
     </row>
     <row r="35" spans="1:16">
       <c r="A35">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B35" t="s">
         <v>67</v>
       </c>
-      <c r="D35">
-        <v>1465</v>
-      </c>
-      <c r="E35" s="2">
-        <v>46104</v>
-      </c>
-      <c r="F35" t="s">
-        <v>83</v>
-      </c>
-      <c r="H35" s="2">
-        <v>46106</v>
-      </c>
-      <c r="I35">
-        <v>27801.11</v>
-      </c>
-      <c r="J35" t="s">
-        <v>128</v>
-      </c>
-      <c r="K35">
-        <v>27801.11</v>
+      <c r="G35" t="s">
+        <v>100</v>
+      </c>
+      <c r="L35">
+        <v>4192.68</v>
       </c>
       <c r="M35" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="N35" t="s">
-        <v>131</v>
-      </c>
-      <c r="P35">
-        <v>1500000</v>
+        <v>135</v>
       </c>
     </row>
     <row r="36" spans="1:16">
@@ -2393,36 +2364,74 @@
         <v>68</v>
       </c>
       <c r="D36">
+        <v>1465</v>
+      </c>
+      <c r="E36" s="1">
+        <v>46104</v>
+      </c>
+      <c r="F36" t="s">
+        <v>84</v>
+      </c>
+      <c r="H36" s="1">
+        <v>46106</v>
+      </c>
+      <c r="I36">
+        <v>27801.11</v>
+      </c>
+      <c r="J36" t="s">
+        <v>130</v>
+      </c>
+      <c r="K36">
+        <v>27801.11</v>
+      </c>
+      <c r="M36" t="s">
+        <v>132</v>
+      </c>
+      <c r="N36" t="s">
+        <v>133</v>
+      </c>
+      <c r="P36">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16">
+      <c r="A37">
+        <v>3</v>
+      </c>
+      <c r="B37" t="s">
+        <v>69</v>
+      </c>
+      <c r="D37">
         <v>1882</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E37" s="1">
         <v>46199</v>
       </c>
-      <c r="F36" t="s">
-        <v>97</v>
-      </c>
-      <c r="H36" s="2">
+      <c r="F37" t="s">
+        <v>99</v>
+      </c>
+      <c r="H37" s="1">
         <v>46233</v>
       </c>
-      <c r="I36">
+      <c r="I37">
         <v>58868.35</v>
       </c>
-      <c r="J36" t="s">
-        <v>127</v>
-      </c>
-      <c r="K36">
+      <c r="J37" t="s">
+        <v>129</v>
+      </c>
+      <c r="K37">
         <v>58868.35</v>
       </c>
-      <c r="M36" t="s">
-        <v>130</v>
-      </c>
-      <c r="N36" t="s">
+      <c r="M37" t="s">
         <v>132</v>
       </c>
-      <c r="O36">
+      <c r="N37" t="s">
+        <v>134</v>
+      </c>
+      <c r="O37">
         <v>0.01</v>
       </c>
-      <c r="P36">
+      <c r="P37">
         <v>2364771.06</v>
       </c>
     </row>
@@ -2437,25 +2446,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="C1" t="s">
         <v>137</v>
+      </c>
+      <c r="D1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E1" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B2">
         <v>1000</v>
@@ -2466,7 +2475,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B3">
         <v>52250.04</v>
@@ -2477,7 +2486,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B4">
         <v>881914.1800000001</v>
@@ -2488,7 +2497,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B5">
         <v>750000</v>
@@ -2499,7 +2508,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B6">
         <v>949835.78</v>
@@ -2510,7 +2519,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B7">
         <v>524584.95</v>
@@ -2521,7 +2530,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B8">
         <v>211614.23</v>
@@ -2532,7 +2541,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B9">
         <v>2391157.41</v>
@@ -2543,7 +2552,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B10">
         <v>618154.38</v>
@@ -2554,7 +2563,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B11">
         <v>1600334.09</v>
@@ -2565,7 +2574,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B12">
         <v>2364771.06</v>
@@ -2576,7 +2585,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B13">
         <v>968237.39</v>
@@ -2587,7 +2596,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B14">
         <v>1011677.95</v>
@@ -2598,7 +2607,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B15">
         <v>1580293.02</v>
@@ -2609,7 +2618,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2620,7 +2629,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B17">
         <v>63746.85</v>
@@ -2631,7 +2640,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B18">
         <v>947931.1</v>
@@ -2642,7 +2651,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B19">
         <v>259790.57</v>
@@ -2653,7 +2662,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B20">
         <v>170479.3</v>
@@ -2664,7 +2673,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B21">
         <v>1500000</v>
@@ -2675,7 +2684,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B22">
         <v>1000001.64</v>
@@ -2686,7 +2695,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B23">
         <v>68405.66</v>
@@ -2697,7 +2706,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B24">
         <v>1157673.06</v>
@@ -2708,7 +2717,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B25">
         <v>34065.36</v>
@@ -2719,7 +2728,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B26">
         <v>1464737.79</v>
@@ -2730,7 +2739,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B27">
         <v>1912292.52</v>
@@ -2741,7 +2750,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -2752,7 +2761,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B29">
         <v>624166.14</v>
@@ -2763,7 +2772,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B30">
         <v>18462.36</v>
@@ -2774,7 +2783,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B31">
         <v>0</v>
@@ -2785,7 +2794,7 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B32">
         <v>0</v>
@@ -2796,7 +2805,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B33">
         <v>236343.68</v>
@@ -2807,7 +2816,7 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B34">
         <v>0</v>
@@ -2818,7 +2827,7 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B35">
         <v>0</v>
@@ -2829,7 +2838,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B36">
         <v>0</v>
@@ -2840,7 +2849,7 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -2851,7 +2860,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B38">
         <v>0</v>
@@ -2862,7 +2871,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -2873,7 +2882,7 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B40">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (19/10/2026 13:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="204">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -524,6 +524,114 @@
   </si>
   <si>
     <t>2026NE001551</t>
+  </si>
+  <si>
+    <t>661.0</t>
+  </si>
+  <si>
+    <t>620.0</t>
+  </si>
+  <si>
+    <t>594.0</t>
+  </si>
+  <si>
+    <t>634.0</t>
+  </si>
+  <si>
+    <t>402.0</t>
+  </si>
+  <si>
+    <t>447.0</t>
+  </si>
+  <si>
+    <t>15.0</t>
+  </si>
+  <si>
+    <t>28.0</t>
+  </si>
+  <si>
+    <t>29.0</t>
+  </si>
+  <si>
+    <t>691.0</t>
+  </si>
+  <si>
+    <t>529.0</t>
+  </si>
+  <si>
+    <t>33.0</t>
+  </si>
+  <si>
+    <t>660.0</t>
+  </si>
+  <si>
+    <t>677.0</t>
+  </si>
+  <si>
+    <t>48.0</t>
+  </si>
+  <si>
+    <t>40.0</t>
+  </si>
+  <si>
+    <t>1882.0</t>
+  </si>
+  <si>
+    <t>5.0</t>
+  </si>
+  <si>
+    <t>696.0</t>
+  </si>
+  <si>
+    <t>688.0</t>
+  </si>
+  <si>
+    <t>748.0</t>
+  </si>
+  <si>
+    <t>728.0</t>
+  </si>
+  <si>
+    <t>715.0</t>
+  </si>
+  <si>
+    <t>704.0</t>
+  </si>
+  <si>
+    <t>1465.0</t>
+  </si>
+  <si>
+    <t>10.0</t>
+  </si>
+  <si>
+    <t>1360.0</t>
+  </si>
+  <si>
+    <t>822.0</t>
+  </si>
+  <si>
+    <t>1278.0</t>
+  </si>
+  <si>
+    <t>66.0</t>
+  </si>
+  <si>
+    <t>2245.0</t>
+  </si>
+  <si>
+    <t>2243.0</t>
+  </si>
+  <si>
+    <t>2244.0</t>
+  </si>
+  <si>
+    <t>56.0</t>
+  </si>
+  <si>
+    <t>71.0</t>
+  </si>
+  <si>
+    <t>/ /</t>
   </si>
 </sst>
 </file>
@@ -533,8 +641,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -550,7 +666,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -558,12 +674,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -863,37 +997,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -943,58 +1077,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1011,13 +1145,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1052,13 +1186,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1093,13 +1227,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1134,13 +1268,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1175,13 +1309,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1219,13 +1353,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1260,13 +1394,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>79</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1301,13 +1435,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>80</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1339,13 +1473,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1380,13 +1514,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1421,13 +1555,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>83</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1462,13 +1596,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1500,13 +1634,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1541,13 +1675,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>86</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1582,13 +1716,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1623,13 +1757,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>87</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1664,13 +1798,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>87</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1705,13 +1839,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>88</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1746,13 +1880,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>89</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="I20">
@@ -1784,13 +1918,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>90</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1825,7 +1959,7 @@
       <c r="D22">
         <v>71</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>46309</v>
       </c>
       <c r="F22" t="s">
@@ -1841,7 +1975,10 @@
         <v>134</v>
       </c>
       <c r="O22">
-        <v>1648399.2</v>
+        <v>82891.44</v>
+      </c>
+      <c r="P22">
+        <v>1565507.76</v>
       </c>
     </row>
     <row r="23" spans="1:16">
@@ -1854,13 +1991,13 @@
       <c r="D23">
         <v>402</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45791</v>
       </c>
       <c r="F23" t="s">
         <v>92</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45834</v>
       </c>
       <c r="I23">
@@ -1895,13 +2032,13 @@
       <c r="D24">
         <v>447</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45814</v>
       </c>
       <c r="F24" t="s">
         <v>93</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45955</v>
       </c>
       <c r="I24">
@@ -1939,13 +2076,13 @@
       <c r="D25">
         <v>529</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45853</v>
       </c>
       <c r="F25" t="s">
         <v>94</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45939</v>
       </c>
       <c r="I25">
@@ -1983,13 +2120,13 @@
       <c r="D26">
         <v>691</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45910</v>
       </c>
       <c r="F26" t="s">
         <v>94</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45941</v>
       </c>
       <c r="I26">
@@ -2027,13 +2164,13 @@
       <c r="D27">
         <v>677</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45904</v>
       </c>
       <c r="F27" t="s">
         <v>76</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2068,13 +2205,13 @@
       <c r="D28">
         <v>278</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46008</v>
       </c>
       <c r="F28" t="s">
         <v>95</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46066</v>
       </c>
       <c r="I28">
@@ -2109,13 +2246,13 @@
       <c r="D29">
         <v>748</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45930</v>
       </c>
       <c r="F29" t="s">
         <v>96</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45935</v>
       </c>
       <c r="I29">
@@ -2150,13 +2287,13 @@
       <c r="D30">
         <v>822</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>45968</v>
       </c>
       <c r="F30" t="s">
         <v>97</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>45935</v>
       </c>
       <c r="I30">
@@ -2191,13 +2328,13 @@
       <c r="D31">
         <v>360</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46043</v>
       </c>
       <c r="F31" t="s">
         <v>84</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46075</v>
       </c>
       <c r="I31">
@@ -2229,13 +2366,13 @@
       <c r="D32">
         <v>2243</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>98</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2267,13 +2404,13 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>98</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2305,13 +2442,13 @@
       <c r="B34" t="s">
         <v>66</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46289</v>
       </c>
       <c r="F34" t="s">
         <v>98</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46325</v>
       </c>
       <c r="I34">
@@ -2366,13 +2503,13 @@
       <c r="D36">
         <v>1465</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46104</v>
       </c>
       <c r="F36" t="s">
         <v>84</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46106</v>
       </c>
       <c r="I36">
@@ -2404,13 +2541,13 @@
       <c r="D37">
         <v>1882</v>
       </c>
-      <c r="E37" s="1">
+      <c r="E37" s="2">
         <v>46199</v>
       </c>
       <c r="F37" t="s">
         <v>99</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46233</v>
       </c>
       <c r="I37">
@@ -2442,23 +2579,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>139</v>
       </c>
     </row>
@@ -2786,10 +2923,10 @@
         <v>158</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>1447765.18</v>
       </c>
       <c r="C31">
-        <v>1530656.62</v>
+        <v>82891.44</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -2885,10 +3022,290 @@
         <v>167</v>
       </c>
       <c r="B40">
-        <v>0</v>
+        <v>117742.58</v>
       </c>
       <c r="C40">
-        <v>117742.58</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>168</v>
+      </c>
+      <c r="B41" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>169</v>
+      </c>
+      <c r="B42" s="2">
+        <v>45813</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>170</v>
+      </c>
+      <c r="B43" s="2">
+        <v>45813</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>171</v>
+      </c>
+      <c r="B44" s="2">
+        <v>45842</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>172</v>
+      </c>
+      <c r="B45" s="2">
+        <v>45862</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>173</v>
+      </c>
+      <c r="B46" s="2">
+        <v>45993</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
+        <v>174</v>
+      </c>
+      <c r="B47" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>175</v>
+      </c>
+      <c r="B48" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
+        <v>176</v>
+      </c>
+      <c r="B49" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>177</v>
+      </c>
+      <c r="B50" s="2">
+        <v>45937</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" t="s">
+        <v>178</v>
+      </c>
+      <c r="B51" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" t="s">
+        <v>179</v>
+      </c>
+      <c r="B52" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" t="s">
+        <v>180</v>
+      </c>
+      <c r="B53" s="2">
+        <v>45889</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" t="s">
+        <v>181</v>
+      </c>
+      <c r="B54" s="2">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" t="s">
+        <v>182</v>
+      </c>
+      <c r="B55" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" t="s">
+        <v>183</v>
+      </c>
+      <c r="B56" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" t="s">
+        <v>184</v>
+      </c>
+      <c r="B57" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" t="s">
+        <v>185</v>
+      </c>
+      <c r="B58" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" t="s">
+        <v>186</v>
+      </c>
+      <c r="B59" s="2">
+        <v>45980</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
+        <v>187</v>
+      </c>
+      <c r="B60" s="2">
+        <v>45930</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" t="s">
+        <v>188</v>
+      </c>
+      <c r="B61" s="2">
+        <v>45993</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" t="s">
+        <v>189</v>
+      </c>
+      <c r="B62" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" t="s">
+        <v>190</v>
+      </c>
+      <c r="B63" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" t="s">
+        <v>191</v>
+      </c>
+      <c r="B64" s="2">
+        <v>45993</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" t="s">
+        <v>192</v>
+      </c>
+      <c r="B65" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" t="s">
+        <v>193</v>
+      </c>
+      <c r="B66" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" t="s">
+        <v>194</v>
+      </c>
+      <c r="B67" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" t="s">
+        <v>195</v>
+      </c>
+      <c r="B68" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" t="s">
+        <v>196</v>
+      </c>
+      <c r="B69" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" t="s">
+        <v>197</v>
+      </c>
+      <c r="B70" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" t="s">
+        <v>198</v>
+      </c>
+      <c r="B71" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" t="s">
+        <v>199</v>
+      </c>
+      <c r="B72" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" t="s">
+        <v>200</v>
+      </c>
+      <c r="B73" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" t="s">
+        <v>201</v>
+      </c>
+      <c r="B74" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" t="s">
+        <v>202</v>
+      </c>
+      <c r="B75" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (19/10/2026 13:40)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="206">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -255,7 +255,7 @@
 2025NE000774</t>
   </si>
   <si>
-    <t>2025NE000843, 2025NE001200</t>
+    <t>2025NE001598</t>
   </si>
   <si>
     <t>2025NE001200</t>
@@ -277,7 +277,7 @@
     <t>2025NE001823</t>
   </si>
   <si>
-    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
+    <t>2025NE000770</t>
   </si>
   <si>
     <t>2025NE000770, 2025NE001627</t>
@@ -286,6 +286,12 @@
     <t>2025NE000770, 2025NE001065, 2025NE001627</t>
   </si>
   <si>
+    <t>2025NE000770, 2025NE001823</t>
+  </si>
+  <si>
+    <t>2025NE001065</t>
+  </si>
+  <si>
     <t>2025NE001065, 2026NE000330</t>
   </si>
   <si>
@@ -304,9 +310,6 @@
     <t>2025NE000770, 2025NE001200</t>
   </si>
   <si>
-    <t>2025NE000770</t>
-  </si>
-  <si>
     <t>2025NE002200</t>
   </si>
   <si>
@@ -319,9 +322,6 @@
     <t>2026NE000330</t>
   </si>
   <si>
-    <t>2025NE001065</t>
-  </si>
-  <si>
     <t>AGUARDANDO ITENS</t>
   </si>
   <si>
@@ -361,12 +361,15 @@
     <t>2026NP401035</t>
   </si>
   <si>
+    <t>2026NP401856</t>
+  </si>
+  <si>
+    <t>2026NP401762</t>
+  </si>
+  <si>
     <t>2026NP402272</t>
   </si>
   <si>
-    <t>2026NP401762</t>
-  </si>
-  <si>
     <t>2026NP402148</t>
   </si>
   <si>
@@ -382,6 +385,9 @@
     <t>2026NP403583</t>
   </si>
   <si>
+    <t>Faturado</t>
+  </si>
+  <si>
     <t>2025NP002620</t>
   </si>
   <si>
@@ -409,7 +415,10 @@
     <t>2026NP400445</t>
   </si>
   <si>
-    <t>Faturado</t>
+    <t>2026NP403699</t>
+  </si>
+  <si>
+    <t>2026NP403700</t>
   </si>
   <si>
     <t>2026NP401058</t>
@@ -461,9 +470,6 @@
   </si>
   <si>
     <t>2025NE000774</t>
-  </si>
-  <si>
-    <t>2025NE001598</t>
   </si>
   <si>
     <t>2025NE001627</t>
@@ -1164,10 +1170,10 @@
         <v>748504.24</v>
       </c>
       <c r="M2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P2">
         <v>881914.1800000001</v>
@@ -1205,10 +1211,10 @@
         <v>1110378.24</v>
       </c>
       <c r="M3" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P3">
         <v>2634000</v>
@@ -1246,10 +1252,10 @@
         <v>974557.12</v>
       </c>
       <c r="M4" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P4">
         <v>1686034.96</v>
@@ -1287,10 +1293,10 @@
         <v>1402001.34</v>
       </c>
       <c r="M5" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N5" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P5">
         <v>1600334.09</v>
@@ -1328,10 +1334,10 @@
         <v>1223702.3</v>
       </c>
       <c r="M6" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O6">
         <v>0.02</v>
@@ -1372,13 +1378,13 @@
         <v>1011677.95</v>
       </c>
       <c r="M7" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N7" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P7">
-        <v>2568571.48</v>
+        <v>1011677.95</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -1401,7 +1407,7 @@
         <v>79</v>
       </c>
       <c r="H8" s="2">
-        <v>45938</v>
+        <v>45955</v>
       </c>
       <c r="I8">
         <v>896744.0600000001</v>
@@ -1413,10 +1419,10 @@
         <v>896744.0600000001</v>
       </c>
       <c r="M8" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P8">
         <v>968237.39</v>
@@ -1454,10 +1460,10 @@
         <v>919329.0600000001</v>
       </c>
       <c r="M9" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P9">
         <v>1947932.74</v>
@@ -1471,7 +1477,7 @@
         <v>42</v>
       </c>
       <c r="D10">
-        <v>705</v>
+        <v>715</v>
       </c>
       <c r="E10" s="2">
         <v>45972</v>
@@ -1492,10 +1498,10 @@
         <v>1157009.26</v>
       </c>
       <c r="M10" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N10" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P10">
         <v>3105605.8</v>
@@ -1533,10 +1539,10 @@
         <v>1214597.952</v>
       </c>
       <c r="M11" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N11" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P11">
         <v>2096487.74</v>
@@ -1553,7 +1559,7 @@
         <v>70</v>
       </c>
       <c r="D12">
-        <v>278</v>
+        <v>5</v>
       </c>
       <c r="E12" s="2">
         <v>46042</v>
@@ -1562,22 +1568,22 @@
         <v>83</v>
       </c>
       <c r="H12" s="2">
-        <v>46074</v>
+        <v>46073</v>
       </c>
       <c r="I12">
-        <v>967082.09</v>
+        <v>967082.9</v>
       </c>
       <c r="J12" t="s">
         <v>111</v>
       </c>
       <c r="K12">
-        <v>967082.09</v>
+        <v>967082.9</v>
       </c>
       <c r="M12" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N12" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O12">
         <v>0.01</v>
@@ -1615,10 +1621,10 @@
         <v>719561.08</v>
       </c>
       <c r="M13" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N13" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P13">
         <v>1500000</v>
@@ -1653,16 +1659,16 @@
         <v>885881.08</v>
       </c>
       <c r="M14" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N14" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O14">
-        <v>34065.36</v>
+        <v>0.01</v>
       </c>
       <c r="P14">
-        <v>3080293.02</v>
+        <v>2391157.41</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -1694,10 +1700,10 @@
         <v>1350542.52</v>
       </c>
       <c r="M15" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N15" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O15">
         <v>0.01</v>
@@ -1729,16 +1735,16 @@
         <v>1108954.435833333</v>
       </c>
       <c r="J16" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K16">
         <v>1108954.435833333</v>
       </c>
       <c r="M16" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N16" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O16">
         <v>0.02</v>
@@ -1761,7 +1767,7 @@
         <v>46149</v>
       </c>
       <c r="F17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H17" s="2">
         <v>46185</v>
@@ -1770,22 +1776,22 @@
         <v>218206.1</v>
       </c>
       <c r="J17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K17">
         <v>218206.1</v>
       </c>
       <c r="M17" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N17" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O17">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="P17">
-        <v>6336221.49</v>
+        <v>3891157.41</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -1799,34 +1805,34 @@
         <v>40</v>
       </c>
       <c r="E18" s="2">
-        <v>46156</v>
+        <v>46188</v>
       </c>
       <c r="F18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H18" s="2">
-        <v>46191</v>
+        <v>46219</v>
       </c>
       <c r="I18">
         <v>1549250.84</v>
       </c>
       <c r="J18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K18">
         <v>1549250.84</v>
       </c>
       <c r="M18" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N18" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O18">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="P18">
-        <v>6336221.49</v>
+        <v>2364771.06</v>
       </c>
     </row>
     <row r="19" spans="1:16">
@@ -1843,25 +1849,25 @@
         <v>46230</v>
       </c>
       <c r="F19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
-        <v>1340865.98</v>
+        <v>1340863.42</v>
       </c>
       <c r="J19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K19">
-        <v>1340865.98</v>
+        <v>1340863.42</v>
       </c>
       <c r="M19" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N19" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O19">
         <v>306142.72</v>
@@ -1878,31 +1884,31 @@
         <v>52</v>
       </c>
       <c r="D20">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E20" s="2">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="F20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H20" s="2">
-        <v>46284</v>
+        <v>46292</v>
       </c>
       <c r="I20">
         <v>1629834.48</v>
       </c>
       <c r="J20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K20">
         <v>1629834.48</v>
       </c>
       <c r="M20" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N20" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P20">
         <v>1912292.52</v>
@@ -1922,7 +1928,7 @@
         <v>46280</v>
       </c>
       <c r="F21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H21" s="2">
         <v>46312</v>
@@ -1931,16 +1937,16 @@
         <v>1675964.21</v>
       </c>
       <c r="J21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K21">
         <v>1675964.21</v>
       </c>
       <c r="M21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N21" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O21">
         <v>306142.71</v>
@@ -1960,19 +1966,25 @@
         <v>71</v>
       </c>
       <c r="E22" s="2">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="F22" t="s">
-        <v>91</v>
+        <v>93</v>
+      </c>
+      <c r="H22" s="2">
+        <v>46342</v>
       </c>
       <c r="I22">
         <v>1565507.76</v>
       </c>
+      <c r="J22" t="s">
+        <v>121</v>
+      </c>
       <c r="M22" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="N22" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="O22">
         <v>82891.44</v>
@@ -1995,7 +2007,7 @@
         <v>45791</v>
       </c>
       <c r="F23" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H23" s="2">
         <v>45834</v>
@@ -2004,16 +2016,16 @@
         <v>188246.17</v>
       </c>
       <c r="J23" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="K23">
         <v>188246.17</v>
       </c>
       <c r="M23" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N23" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P23">
         <v>211614.23</v>
@@ -2036,7 +2048,7 @@
         <v>45814</v>
       </c>
       <c r="F24" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H24" s="2">
         <v>45955</v>
@@ -2045,16 +2057,16 @@
         <v>112720.77</v>
       </c>
       <c r="J24" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="K24">
         <v>112720.77</v>
       </c>
       <c r="M24" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N24" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O24">
         <v>0.01</v>
@@ -2080,7 +2092,7 @@
         <v>45853</v>
       </c>
       <c r="F25" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="H25" s="2">
         <v>45939</v>
@@ -2089,16 +2101,16 @@
         <v>378307.61</v>
       </c>
       <c r="J25" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="K25">
         <v>378307.61</v>
       </c>
       <c r="M25" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N25" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O25">
         <v>0.01</v>
@@ -2124,25 +2136,25 @@
         <v>45910</v>
       </c>
       <c r="F26" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="H26" s="2">
         <v>45941</v>
       </c>
       <c r="I26">
-        <v>3315.047100000025</v>
+        <v>3315.06</v>
       </c>
       <c r="J26" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="K26">
-        <v>3315.04710000003</v>
+        <v>3315.06</v>
       </c>
       <c r="M26" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N26" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="O26">
         <v>0.01</v>
@@ -2177,16 +2189,16 @@
         <v>198332.75</v>
       </c>
       <c r="J27" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="K27">
         <v>198332.75</v>
       </c>
       <c r="M27" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N27" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P27">
         <v>1600334.09</v>
@@ -2203,13 +2215,13 @@
         <v>40</v>
       </c>
       <c r="D28">
-        <v>278</v>
+        <v>1278</v>
       </c>
       <c r="E28" s="2">
         <v>46008</v>
       </c>
       <c r="F28" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H28" s="2">
         <v>46066</v>
@@ -2218,16 +2230,16 @@
         <v>1528.62</v>
       </c>
       <c r="J28" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="K28">
         <v>1528.62</v>
       </c>
       <c r="M28" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N28" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P28">
         <v>1157673.06</v>
@@ -2250,25 +2262,25 @@
         <v>45930</v>
       </c>
       <c r="F29" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H29" s="2">
-        <v>45935</v>
+        <v>45991</v>
       </c>
       <c r="I29">
         <v>38718.58</v>
       </c>
       <c r="J29" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="K29">
         <v>38718.58</v>
       </c>
       <c r="M29" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N29" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P29">
         <v>63746.85</v>
@@ -2291,25 +2303,25 @@
         <v>45968</v>
       </c>
       <c r="F30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H30" s="2">
-        <v>45935</v>
+        <v>46001</v>
       </c>
       <c r="I30">
         <v>133124.11</v>
       </c>
       <c r="J30" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K30">
         <v>133124.11</v>
       </c>
       <c r="M30" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N30" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P30">
         <v>1000001.64</v>
@@ -2326,7 +2338,7 @@
         <v>252</v>
       </c>
       <c r="D31">
-        <v>360</v>
+        <v>1360</v>
       </c>
       <c r="E31" s="2">
         <v>46043</v>
@@ -2341,16 +2353,16 @@
         <v>11372.9</v>
       </c>
       <c r="J31" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="K31">
         <v>11372.9</v>
       </c>
       <c r="M31" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N31" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P31">
         <v>1500000</v>
@@ -2370,7 +2382,7 @@
         <v>46289</v>
       </c>
       <c r="F32" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H32" s="2">
         <v>46325</v>
@@ -2379,16 +2391,16 @@
         <v>15854.78</v>
       </c>
       <c r="J32" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K32">
         <v>15854.78</v>
       </c>
       <c r="M32" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N32" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="O32">
         <v>306142.71</v>
@@ -2404,11 +2416,14 @@
       <c r="B33" t="s">
         <v>65</v>
       </c>
+      <c r="D33">
+        <v>2245</v>
+      </c>
       <c r="E33" s="2">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H33" s="2">
         <v>46325</v>
@@ -2417,16 +2432,16 @@
         <v>42229.72325</v>
       </c>
       <c r="J33" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="K33">
         <v>42229.72325</v>
       </c>
       <c r="M33" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N33" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="O33">
         <v>306142.71</v>
@@ -2442,11 +2457,14 @@
       <c r="B34" t="s">
         <v>66</v>
       </c>
+      <c r="D34">
+        <v>2244</v>
+      </c>
       <c r="E34" s="2">
         <v>46289</v>
       </c>
       <c r="F34" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H34" s="2">
         <v>46325</v>
@@ -2455,16 +2473,16 @@
         <v>48857.39550000001</v>
       </c>
       <c r="J34" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="K34">
         <v>48857.39550000001</v>
       </c>
       <c r="M34" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N34" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="O34">
         <v>306142.71</v>
@@ -2487,10 +2505,10 @@
         <v>4192.68</v>
       </c>
       <c r="M35" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N35" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="36" spans="1:16">
@@ -2504,7 +2522,7 @@
         <v>1465</v>
       </c>
       <c r="E36" s="2">
-        <v>46104</v>
+        <v>46076</v>
       </c>
       <c r="F36" t="s">
         <v>84</v>
@@ -2516,16 +2534,16 @@
         <v>27801.11</v>
       </c>
       <c r="J36" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="K36">
         <v>27801.11</v>
       </c>
       <c r="M36" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N36" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="P36">
         <v>1500000</v>
@@ -2545,31 +2563,31 @@
         <v>46199</v>
       </c>
       <c r="F37" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="H37" s="2">
         <v>46233</v>
       </c>
       <c r="I37">
-        <v>58868.35</v>
+        <v>58868.34</v>
       </c>
       <c r="J37" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="K37">
-        <v>58868.35</v>
+        <v>58868.34</v>
       </c>
       <c r="M37" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N37" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="O37">
-        <v>0.01</v>
+        <v>306142.72</v>
       </c>
       <c r="P37">
-        <v>2364771.06</v>
+        <v>3829508.85</v>
       </c>
     </row>
   </sheetData>
@@ -2584,24 +2602,24 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B2">
         <v>1000</v>
@@ -2612,7 +2630,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B3">
         <v>52250.04</v>
@@ -2623,7 +2641,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B4">
         <v>881914.1800000001</v>
@@ -2634,7 +2652,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B5">
         <v>750000</v>
@@ -2645,7 +2663,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B6">
         <v>949835.78</v>
@@ -2656,7 +2674,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B7">
         <v>524584.95</v>
@@ -2667,7 +2685,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B8">
         <v>211614.23</v>
@@ -2678,7 +2696,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="B9">
         <v>2391157.41</v>
@@ -2689,7 +2707,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B10">
         <v>618154.38</v>
@@ -2711,7 +2729,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="B12">
         <v>2364771.06</v>
@@ -2733,7 +2751,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>147</v>
+        <v>78</v>
       </c>
       <c r="B14">
         <v>1011677.95</v>
@@ -2744,7 +2762,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B15">
         <v>1580293.02</v>
@@ -2755,7 +2773,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2766,7 +2784,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B17">
         <v>63746.85</v>
@@ -2777,7 +2795,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B18">
         <v>947931.1</v>
@@ -2788,7 +2806,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B19">
         <v>259790.57</v>
@@ -2799,7 +2817,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B20">
         <v>170479.3</v>
@@ -2821,7 +2839,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B22">
         <v>1000001.64</v>
@@ -2832,7 +2850,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B23">
         <v>68405.66</v>
@@ -2843,7 +2861,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B24">
         <v>1157673.06</v>
@@ -2854,7 +2872,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B25">
         <v>34065.36</v>
@@ -2865,7 +2883,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B26">
         <v>1464737.79</v>
@@ -2876,7 +2894,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B27">
         <v>1912292.52</v>
@@ -2887,7 +2905,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -2898,7 +2916,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B29">
         <v>624166.14</v>
@@ -2909,7 +2927,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B30">
         <v>18462.36</v>
@@ -2920,7 +2938,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B31">
         <v>1447765.18</v>
@@ -2931,7 +2949,7 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B32">
         <v>0</v>
@@ -2942,7 +2960,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B33">
         <v>236343.68</v>
@@ -2953,7 +2971,7 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B34">
         <v>0</v>
@@ -2964,7 +2982,7 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B35">
         <v>0</v>
@@ -2975,7 +2993,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B36">
         <v>0</v>
@@ -2986,7 +3004,7 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -2997,7 +3015,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B38">
         <v>0</v>
@@ -3008,7 +3026,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -3019,7 +3037,7 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B40">
         <v>117742.58</v>
@@ -3030,15 +3048,15 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B41" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B42" s="2">
         <v>45813</v>
@@ -3046,7 +3064,7 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B43" s="2">
         <v>45813</v>
@@ -3054,7 +3072,7 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B44" s="2">
         <v>45842</v>
@@ -3062,7 +3080,7 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B45" s="2">
         <v>45862</v>
@@ -3070,7 +3088,7 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B46" s="2">
         <v>45993</v>
@@ -3078,31 +3096,31 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B47" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B48" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B49" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B50" s="2">
         <v>45937</v>
@@ -3110,23 +3128,23 @@
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B51" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B52" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B53" s="2">
         <v>45889</v>
@@ -3134,7 +3152,7 @@
     </row>
     <row r="54" spans="1:2">
       <c r="A54" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B54" s="2">
         <v>45931</v>
@@ -3142,39 +3160,39 @@
     </row>
     <row r="55" spans="1:2">
       <c r="A55" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B55" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B56" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B57" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B58" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B59" s="2">
         <v>45980</v>
@@ -3182,7 +3200,7 @@
     </row>
     <row r="60" spans="1:2">
       <c r="A60" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B60" s="2">
         <v>45930</v>
@@ -3190,7 +3208,7 @@
     </row>
     <row r="61" spans="1:2">
       <c r="A61" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B61" s="2">
         <v>45993</v>
@@ -3198,23 +3216,23 @@
     </row>
     <row r="62" spans="1:2">
       <c r="A62" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B62" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B63" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B64" s="2">
         <v>45993</v>
@@ -3222,90 +3240,90 @@
     </row>
     <row r="65" spans="1:2">
       <c r="A65" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B65" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B66" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B67" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B68" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B69" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B70" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B71" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B72" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B73" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B74" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B75" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (19/10/2026 13:44)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -1057,16 +1057,16 @@
         <v>91651597.37</v>
       </c>
       <c r="G2">
-        <v>72543679.31999999</v>
+        <v>60769048.35</v>
       </c>
       <c r="H2">
-        <v>19107918.05</v>
+        <v>30882549.02</v>
       </c>
       <c r="I2">
-        <v>8248487.61</v>
+        <v>24929428.27</v>
       </c>
       <c r="J2">
-        <v>10859430.44</v>
+        <v>5953120.75</v>
       </c>
       <c r="K2" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (19/10/2026 14:26)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -647,16 +647,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -672,7 +664,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -680,30 +672,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1003,37 +977,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1083,58 +1057,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1151,13 +1125,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1192,13 +1166,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1233,13 +1207,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1274,13 +1248,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1315,13 +1289,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1359,13 +1333,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1400,13 +1374,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>79</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45955</v>
       </c>
       <c r="I8">
@@ -1441,13 +1415,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>80</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1479,13 +1453,13 @@
       <c r="D10">
         <v>715</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1520,13 +1494,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1561,13 +1535,13 @@
       <c r="D12">
         <v>5</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>83</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46073</v>
       </c>
       <c r="I12">
@@ -1602,13 +1576,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1640,13 +1614,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1681,13 +1655,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>86</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1722,13 +1696,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1763,13 +1737,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>88</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1804,13 +1778,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46188</v>
       </c>
       <c r="F18" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46219</v>
       </c>
       <c r="I18">
@@ -1845,13 +1819,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>90</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1886,13 +1860,13 @@
       <c r="D20">
         <v>56</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46259</v>
       </c>
       <c r="F20" t="s">
         <v>91</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46292</v>
       </c>
       <c r="I20">
@@ -1924,13 +1898,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1965,13 +1939,13 @@
       <c r="D22">
         <v>71</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>46310</v>
       </c>
       <c r="F22" t="s">
         <v>93</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>46342</v>
       </c>
       <c r="I22">
@@ -2003,13 +1977,13 @@
       <c r="D23">
         <v>402</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45791</v>
       </c>
       <c r="F23" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45834</v>
       </c>
       <c r="I23">
@@ -2044,13 +2018,13 @@
       <c r="D24">
         <v>447</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45814</v>
       </c>
       <c r="F24" t="s">
         <v>95</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45955</v>
       </c>
       <c r="I24">
@@ -2088,13 +2062,13 @@
       <c r="D25">
         <v>529</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45853</v>
       </c>
       <c r="F25" t="s">
         <v>85</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45939</v>
       </c>
       <c r="I25">
@@ -2132,13 +2106,13 @@
       <c r="D26">
         <v>691</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45910</v>
       </c>
       <c r="F26" t="s">
         <v>85</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45941</v>
       </c>
       <c r="I26">
@@ -2176,13 +2150,13 @@
       <c r="D27">
         <v>677</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45904</v>
       </c>
       <c r="F27" t="s">
         <v>76</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2217,13 +2191,13 @@
       <c r="D28">
         <v>1278</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46008</v>
       </c>
       <c r="F28" t="s">
         <v>96</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46066</v>
       </c>
       <c r="I28">
@@ -2258,13 +2232,13 @@
       <c r="D29">
         <v>748</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45930</v>
       </c>
       <c r="F29" t="s">
         <v>97</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45991</v>
       </c>
       <c r="I29">
@@ -2299,13 +2273,13 @@
       <c r="D30">
         <v>822</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>45968</v>
       </c>
       <c r="F30" t="s">
         <v>98</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46001</v>
       </c>
       <c r="I30">
@@ -2340,13 +2314,13 @@
       <c r="D31">
         <v>1360</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46043</v>
       </c>
       <c r="F31" t="s">
         <v>84</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46075</v>
       </c>
       <c r="I31">
@@ -2378,13 +2352,13 @@
       <c r="D32">
         <v>2243</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>99</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2419,13 +2393,13 @@
       <c r="D33">
         <v>2245</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>99</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2460,13 +2434,13 @@
       <c r="D34">
         <v>2244</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46289</v>
       </c>
       <c r="F34" t="s">
         <v>99</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46325</v>
       </c>
       <c r="I34">
@@ -2521,13 +2495,13 @@
       <c r="D36">
         <v>1465</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46076</v>
       </c>
       <c r="F36" t="s">
         <v>84</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46106</v>
       </c>
       <c r="I36">
@@ -2559,13 +2533,13 @@
       <c r="D37">
         <v>1882</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>46199</v>
       </c>
       <c r="F37" t="s">
         <v>90</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46233</v>
       </c>
       <c r="I37">
@@ -2601,19 +2575,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>140</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>141</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>142</v>
       </c>
     </row>
@@ -3058,7 +3032,7 @@
       <c r="A42" t="s">
         <v>171</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="1">
         <v>45813</v>
       </c>
     </row>
@@ -3066,7 +3040,7 @@
       <c r="A43" t="s">
         <v>172</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="1">
         <v>45813</v>
       </c>
     </row>
@@ -3074,7 +3048,7 @@
       <c r="A44" t="s">
         <v>173</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="1">
         <v>45842</v>
       </c>
     </row>
@@ -3082,7 +3056,7 @@
       <c r="A45" t="s">
         <v>174</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="1">
         <v>45862</v>
       </c>
     </row>
@@ -3090,7 +3064,7 @@
       <c r="A46" t="s">
         <v>175</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="1">
         <v>45993</v>
       </c>
     </row>
@@ -3122,7 +3096,7 @@
       <c r="A50" t="s">
         <v>179</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -3146,7 +3120,7 @@
       <c r="A53" t="s">
         <v>182</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="1">
         <v>45889</v>
       </c>
     </row>
@@ -3154,7 +3128,7 @@
       <c r="A54" t="s">
         <v>183</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="1">
         <v>45931</v>
       </c>
     </row>
@@ -3194,7 +3168,7 @@
       <c r="A59" t="s">
         <v>188</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="1">
         <v>45980</v>
       </c>
     </row>
@@ -3202,7 +3176,7 @@
       <c r="A60" t="s">
         <v>189</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="1">
         <v>45930</v>
       </c>
     </row>
@@ -3210,7 +3184,7 @@
       <c r="A61" t="s">
         <v>190</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="1">
         <v>45993</v>
       </c>
     </row>
@@ -3234,7 +3208,7 @@
       <c r="A64" t="s">
         <v>193</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="1">
         <v>45993</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (20/10/2026 12:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -647,8 +647,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -664,7 +672,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -672,12 +680,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -977,37 +1003,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1057,58 +1083,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1125,13 +1151,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1166,13 +1192,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1207,13 +1233,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1248,13 +1274,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1289,13 +1315,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1333,13 +1359,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1374,13 +1400,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>79</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45955</v>
       </c>
       <c r="I8">
@@ -1415,13 +1441,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>80</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1453,13 +1479,13 @@
       <c r="D10">
         <v>715</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1494,13 +1520,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1535,13 +1561,13 @@
       <c r="D12">
         <v>5</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>83</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46073</v>
       </c>
       <c r="I12">
@@ -1576,13 +1602,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1614,13 +1640,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1655,13 +1681,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>86</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1696,13 +1722,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1737,13 +1763,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>88</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1778,13 +1804,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46188</v>
       </c>
       <c r="F18" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46219</v>
       </c>
       <c r="I18">
@@ -1819,13 +1845,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>90</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1860,13 +1886,13 @@
       <c r="D20">
         <v>56</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46259</v>
       </c>
       <c r="F20" t="s">
         <v>91</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46292</v>
       </c>
       <c r="I20">
@@ -1898,13 +1924,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1939,13 +1965,13 @@
       <c r="D22">
         <v>71</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>46310</v>
       </c>
       <c r="F22" t="s">
         <v>93</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>46342</v>
       </c>
       <c r="I22">
@@ -1977,13 +2003,13 @@
       <c r="D23">
         <v>402</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45791</v>
       </c>
       <c r="F23" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45834</v>
       </c>
       <c r="I23">
@@ -2018,13 +2044,13 @@
       <c r="D24">
         <v>447</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45814</v>
       </c>
       <c r="F24" t="s">
         <v>95</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45955</v>
       </c>
       <c r="I24">
@@ -2062,13 +2088,13 @@
       <c r="D25">
         <v>529</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45853</v>
       </c>
       <c r="F25" t="s">
         <v>85</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45939</v>
       </c>
       <c r="I25">
@@ -2106,13 +2132,13 @@
       <c r="D26">
         <v>691</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45910</v>
       </c>
       <c r="F26" t="s">
         <v>85</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45941</v>
       </c>
       <c r="I26">
@@ -2150,13 +2176,13 @@
       <c r="D27">
         <v>677</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45904</v>
       </c>
       <c r="F27" t="s">
         <v>76</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2191,13 +2217,13 @@
       <c r="D28">
         <v>1278</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46008</v>
       </c>
       <c r="F28" t="s">
         <v>96</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46066</v>
       </c>
       <c r="I28">
@@ -2232,13 +2258,13 @@
       <c r="D29">
         <v>748</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45930</v>
       </c>
       <c r="F29" t="s">
         <v>97</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45991</v>
       </c>
       <c r="I29">
@@ -2273,13 +2299,13 @@
       <c r="D30">
         <v>822</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>45968</v>
       </c>
       <c r="F30" t="s">
         <v>98</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46001</v>
       </c>
       <c r="I30">
@@ -2314,13 +2340,13 @@
       <c r="D31">
         <v>1360</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46043</v>
       </c>
       <c r="F31" t="s">
         <v>84</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46075</v>
       </c>
       <c r="I31">
@@ -2352,13 +2378,13 @@
       <c r="D32">
         <v>2243</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>99</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2393,13 +2419,13 @@
       <c r="D33">
         <v>2245</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>99</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2434,13 +2460,13 @@
       <c r="D34">
         <v>2244</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46289</v>
       </c>
       <c r="F34" t="s">
         <v>99</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46325</v>
       </c>
       <c r="I34">
@@ -2495,13 +2521,13 @@
       <c r="D36">
         <v>1465</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46076</v>
       </c>
       <c r="F36" t="s">
         <v>84</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46106</v>
       </c>
       <c r="I36">
@@ -2533,13 +2559,13 @@
       <c r="D37">
         <v>1882</v>
       </c>
-      <c r="E37" s="1">
+      <c r="E37" s="2">
         <v>46199</v>
       </c>
       <c r="F37" t="s">
         <v>90</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46233</v>
       </c>
       <c r="I37">
@@ -2575,19 +2601,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>142</v>
       </c>
     </row>
@@ -3032,7 +3058,7 @@
       <c r="A42" t="s">
         <v>171</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="2">
         <v>45813</v>
       </c>
     </row>
@@ -3040,7 +3066,7 @@
       <c r="A43" t="s">
         <v>172</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="2">
         <v>45813</v>
       </c>
     </row>
@@ -3048,7 +3074,7 @@
       <c r="A44" t="s">
         <v>173</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="2">
         <v>45842</v>
       </c>
     </row>
@@ -3056,7 +3082,7 @@
       <c r="A45" t="s">
         <v>174</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="2">
         <v>45862</v>
       </c>
     </row>
@@ -3064,7 +3090,7 @@
       <c r="A46" t="s">
         <v>175</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="2">
         <v>45993</v>
       </c>
     </row>
@@ -3096,7 +3122,7 @@
       <c r="A50" t="s">
         <v>179</v>
       </c>
-      <c r="B50" s="1">
+      <c r="B50" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -3120,7 +3146,7 @@
       <c r="A53" t="s">
         <v>182</v>
       </c>
-      <c r="B53" s="1">
+      <c r="B53" s="2">
         <v>45889</v>
       </c>
     </row>
@@ -3128,7 +3154,7 @@
       <c r="A54" t="s">
         <v>183</v>
       </c>
-      <c r="B54" s="1">
+      <c r="B54" s="2">
         <v>45931</v>
       </c>
     </row>
@@ -3168,7 +3194,7 @@
       <c r="A59" t="s">
         <v>188</v>
       </c>
-      <c r="B59" s="1">
+      <c r="B59" s="2">
         <v>45980</v>
       </c>
     </row>
@@ -3176,7 +3202,7 @@
       <c r="A60" t="s">
         <v>189</v>
       </c>
-      <c r="B60" s="1">
+      <c r="B60" s="2">
         <v>45930</v>
       </c>
     </row>
@@ -3184,7 +3210,7 @@
       <c r="A61" t="s">
         <v>190</v>
       </c>
-      <c r="B61" s="1">
+      <c r="B61" s="2">
         <v>45993</v>
       </c>
     </row>
@@ -3208,7 +3234,7 @@
       <c r="A64" t="s">
         <v>193</v>
       </c>
-      <c r="B64" s="1">
+      <c r="B64" s="2">
         <v>45993</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (20/10/2026 12:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -647,16 +647,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -672,7 +664,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -680,30 +672,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1003,37 +977,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1083,58 +1057,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1151,13 +1125,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1192,13 +1166,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1233,13 +1207,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1274,13 +1248,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1315,13 +1289,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1359,13 +1333,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1400,13 +1374,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>79</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45955</v>
       </c>
       <c r="I8">
@@ -1441,13 +1415,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>80</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1479,13 +1453,13 @@
       <c r="D10">
         <v>715</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1520,13 +1494,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1561,13 +1535,13 @@
       <c r="D12">
         <v>5</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>83</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46073</v>
       </c>
       <c r="I12">
@@ -1602,13 +1576,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1640,13 +1614,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1681,13 +1655,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>86</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1722,13 +1696,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1763,13 +1737,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>88</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1804,13 +1778,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46188</v>
       </c>
       <c r="F18" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46219</v>
       </c>
       <c r="I18">
@@ -1845,13 +1819,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>90</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1886,13 +1860,13 @@
       <c r="D20">
         <v>56</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46259</v>
       </c>
       <c r="F20" t="s">
         <v>91</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46292</v>
       </c>
       <c r="I20">
@@ -1924,13 +1898,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1965,13 +1939,13 @@
       <c r="D22">
         <v>71</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>46310</v>
       </c>
       <c r="F22" t="s">
         <v>93</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>46342</v>
       </c>
       <c r="I22">
@@ -2003,13 +1977,13 @@
       <c r="D23">
         <v>402</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45791</v>
       </c>
       <c r="F23" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45834</v>
       </c>
       <c r="I23">
@@ -2044,13 +2018,13 @@
       <c r="D24">
         <v>447</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45814</v>
       </c>
       <c r="F24" t="s">
         <v>95</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45955</v>
       </c>
       <c r="I24">
@@ -2088,13 +2062,13 @@
       <c r="D25">
         <v>529</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45853</v>
       </c>
       <c r="F25" t="s">
         <v>85</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45939</v>
       </c>
       <c r="I25">
@@ -2132,13 +2106,13 @@
       <c r="D26">
         <v>691</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45910</v>
       </c>
       <c r="F26" t="s">
         <v>85</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45941</v>
       </c>
       <c r="I26">
@@ -2176,13 +2150,13 @@
       <c r="D27">
         <v>677</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45904</v>
       </c>
       <c r="F27" t="s">
         <v>76</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2217,13 +2191,13 @@
       <c r="D28">
         <v>1278</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46008</v>
       </c>
       <c r="F28" t="s">
         <v>96</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46066</v>
       </c>
       <c r="I28">
@@ -2258,13 +2232,13 @@
       <c r="D29">
         <v>748</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45930</v>
       </c>
       <c r="F29" t="s">
         <v>97</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45991</v>
       </c>
       <c r="I29">
@@ -2299,13 +2273,13 @@
       <c r="D30">
         <v>822</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>45968</v>
       </c>
       <c r="F30" t="s">
         <v>98</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46001</v>
       </c>
       <c r="I30">
@@ -2340,13 +2314,13 @@
       <c r="D31">
         <v>1360</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46043</v>
       </c>
       <c r="F31" t="s">
         <v>84</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46075</v>
       </c>
       <c r="I31">
@@ -2378,13 +2352,13 @@
       <c r="D32">
         <v>2243</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>99</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2419,13 +2393,13 @@
       <c r="D33">
         <v>2245</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>99</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2460,13 +2434,13 @@
       <c r="D34">
         <v>2244</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46289</v>
       </c>
       <c r="F34" t="s">
         <v>99</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46325</v>
       </c>
       <c r="I34">
@@ -2521,13 +2495,13 @@
       <c r="D36">
         <v>1465</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46076</v>
       </c>
       <c r="F36" t="s">
         <v>84</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46106</v>
       </c>
       <c r="I36">
@@ -2559,13 +2533,13 @@
       <c r="D37">
         <v>1882</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>46199</v>
       </c>
       <c r="F37" t="s">
         <v>90</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46233</v>
       </c>
       <c r="I37">
@@ -2601,19 +2575,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>140</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>141</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>142</v>
       </c>
     </row>
@@ -3058,7 +3032,7 @@
       <c r="A42" t="s">
         <v>171</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="1">
         <v>45813</v>
       </c>
     </row>
@@ -3066,7 +3040,7 @@
       <c r="A43" t="s">
         <v>172</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="1">
         <v>45813</v>
       </c>
     </row>
@@ -3074,7 +3048,7 @@
       <c r="A44" t="s">
         <v>173</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="1">
         <v>45842</v>
       </c>
     </row>
@@ -3082,7 +3056,7 @@
       <c r="A45" t="s">
         <v>174</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="1">
         <v>45862</v>
       </c>
     </row>
@@ -3090,7 +3064,7 @@
       <c r="A46" t="s">
         <v>175</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="1">
         <v>45993</v>
       </c>
     </row>
@@ -3122,7 +3096,7 @@
       <c r="A50" t="s">
         <v>179</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -3146,7 +3120,7 @@
       <c r="A53" t="s">
         <v>182</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="1">
         <v>45889</v>
       </c>
     </row>
@@ -3154,7 +3128,7 @@
       <c r="A54" t="s">
         <v>183</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="1">
         <v>45931</v>
       </c>
     </row>
@@ -3194,7 +3168,7 @@
       <c r="A59" t="s">
         <v>188</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="1">
         <v>45980</v>
       </c>
     </row>
@@ -3202,7 +3176,7 @@
       <c r="A60" t="s">
         <v>189</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="1">
         <v>45930</v>
       </c>
     </row>
@@ -3210,7 +3184,7 @@
       <c r="A61" t="s">
         <v>190</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="1">
         <v>45993</v>
       </c>
     </row>
@@ -3234,7 +3208,7 @@
       <c r="A64" t="s">
         <v>193</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="1">
         <v>45993</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (21/10/2026 14:22)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -647,8 +647,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -664,7 +672,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -672,12 +680,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -977,37 +1003,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1057,58 +1083,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1125,13 +1151,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1166,13 +1192,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1207,13 +1233,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1248,13 +1274,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1289,13 +1315,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1333,13 +1359,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1374,13 +1400,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>79</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45955</v>
       </c>
       <c r="I8">
@@ -1415,13 +1441,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>80</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1453,13 +1479,13 @@
       <c r="D10">
         <v>715</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1494,13 +1520,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1535,13 +1561,13 @@
       <c r="D12">
         <v>5</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>83</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46073</v>
       </c>
       <c r="I12">
@@ -1576,13 +1602,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1614,13 +1640,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1655,13 +1681,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>86</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1696,13 +1722,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1737,13 +1763,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>88</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1778,13 +1804,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46188</v>
       </c>
       <c r="F18" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46219</v>
       </c>
       <c r="I18">
@@ -1819,13 +1845,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>90</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1860,13 +1886,13 @@
       <c r="D20">
         <v>56</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46259</v>
       </c>
       <c r="F20" t="s">
         <v>91</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46292</v>
       </c>
       <c r="I20">
@@ -1898,13 +1924,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1939,13 +1965,13 @@
       <c r="D22">
         <v>71</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>46310</v>
       </c>
       <c r="F22" t="s">
         <v>93</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>46342</v>
       </c>
       <c r="I22">
@@ -1977,13 +2003,13 @@
       <c r="D23">
         <v>402</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45791</v>
       </c>
       <c r="F23" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45834</v>
       </c>
       <c r="I23">
@@ -2018,13 +2044,13 @@
       <c r="D24">
         <v>447</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45814</v>
       </c>
       <c r="F24" t="s">
         <v>95</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45955</v>
       </c>
       <c r="I24">
@@ -2062,13 +2088,13 @@
       <c r="D25">
         <v>529</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45853</v>
       </c>
       <c r="F25" t="s">
         <v>85</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45939</v>
       </c>
       <c r="I25">
@@ -2106,13 +2132,13 @@
       <c r="D26">
         <v>691</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45910</v>
       </c>
       <c r="F26" t="s">
         <v>85</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45941</v>
       </c>
       <c r="I26">
@@ -2150,13 +2176,13 @@
       <c r="D27">
         <v>677</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45904</v>
       </c>
       <c r="F27" t="s">
         <v>76</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2191,13 +2217,13 @@
       <c r="D28">
         <v>1278</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46008</v>
       </c>
       <c r="F28" t="s">
         <v>96</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46066</v>
       </c>
       <c r="I28">
@@ -2232,13 +2258,13 @@
       <c r="D29">
         <v>748</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45930</v>
       </c>
       <c r="F29" t="s">
         <v>97</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45991</v>
       </c>
       <c r="I29">
@@ -2273,13 +2299,13 @@
       <c r="D30">
         <v>822</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>45968</v>
       </c>
       <c r="F30" t="s">
         <v>98</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46001</v>
       </c>
       <c r="I30">
@@ -2314,13 +2340,13 @@
       <c r="D31">
         <v>1360</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46043</v>
       </c>
       <c r="F31" t="s">
         <v>84</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46075</v>
       </c>
       <c r="I31">
@@ -2352,13 +2378,13 @@
       <c r="D32">
         <v>2243</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>99</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2393,13 +2419,13 @@
       <c r="D33">
         <v>2245</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>99</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2434,13 +2460,13 @@
       <c r="D34">
         <v>2244</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46289</v>
       </c>
       <c r="F34" t="s">
         <v>99</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46325</v>
       </c>
       <c r="I34">
@@ -2495,13 +2521,13 @@
       <c r="D36">
         <v>1465</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46076</v>
       </c>
       <c r="F36" t="s">
         <v>84</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46106</v>
       </c>
       <c r="I36">
@@ -2533,13 +2559,13 @@
       <c r="D37">
         <v>1882</v>
       </c>
-      <c r="E37" s="1">
+      <c r="E37" s="2">
         <v>46199</v>
       </c>
       <c r="F37" t="s">
         <v>90</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46233</v>
       </c>
       <c r="I37">
@@ -2575,19 +2601,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>142</v>
       </c>
     </row>
@@ -3032,7 +3058,7 @@
       <c r="A42" t="s">
         <v>171</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="2">
         <v>45813</v>
       </c>
     </row>
@@ -3040,7 +3066,7 @@
       <c r="A43" t="s">
         <v>172</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="2">
         <v>45813</v>
       </c>
     </row>
@@ -3048,7 +3074,7 @@
       <c r="A44" t="s">
         <v>173</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="2">
         <v>45842</v>
       </c>
     </row>
@@ -3056,7 +3082,7 @@
       <c r="A45" t="s">
         <v>174</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="2">
         <v>45862</v>
       </c>
     </row>
@@ -3064,7 +3090,7 @@
       <c r="A46" t="s">
         <v>175</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="2">
         <v>45993</v>
       </c>
     </row>
@@ -3096,7 +3122,7 @@
       <c r="A50" t="s">
         <v>179</v>
       </c>
-      <c r="B50" s="1">
+      <c r="B50" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -3120,7 +3146,7 @@
       <c r="A53" t="s">
         <v>182</v>
       </c>
-      <c r="B53" s="1">
+      <c r="B53" s="2">
         <v>45889</v>
       </c>
     </row>
@@ -3128,7 +3154,7 @@
       <c r="A54" t="s">
         <v>183</v>
       </c>
-      <c r="B54" s="1">
+      <c r="B54" s="2">
         <v>45931</v>
       </c>
     </row>
@@ -3168,7 +3194,7 @@
       <c r="A59" t="s">
         <v>188</v>
       </c>
-      <c r="B59" s="1">
+      <c r="B59" s="2">
         <v>45980</v>
       </c>
     </row>
@@ -3176,7 +3202,7 @@
       <c r="A60" t="s">
         <v>189</v>
       </c>
-      <c r="B60" s="1">
+      <c r="B60" s="2">
         <v>45930</v>
       </c>
     </row>
@@ -3184,7 +3210,7 @@
       <c r="A61" t="s">
         <v>190</v>
       </c>
-      <c r="B61" s="1">
+      <c r="B61" s="2">
         <v>45993</v>
       </c>
     </row>
@@ -3208,7 +3234,7 @@
       <c r="A64" t="s">
         <v>193</v>
       </c>
-      <c r="B64" s="1">
+      <c r="B64" s="2">
         <v>45993</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (22/10/2026 12:52)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -647,16 +647,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -672,7 +664,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -680,30 +672,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1003,37 +977,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1083,58 +1057,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1151,13 +1125,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1192,13 +1166,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1233,13 +1207,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1274,13 +1248,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1315,13 +1289,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1359,13 +1333,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1400,13 +1374,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>79</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45955</v>
       </c>
       <c r="I8">
@@ -1441,13 +1415,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>80</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1479,13 +1453,13 @@
       <c r="D10">
         <v>715</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1520,13 +1494,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1561,13 +1535,13 @@
       <c r="D12">
         <v>5</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>83</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46073</v>
       </c>
       <c r="I12">
@@ -1602,13 +1576,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1640,13 +1614,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1681,13 +1655,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>86</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1722,13 +1696,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1763,13 +1737,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>88</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1804,13 +1778,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46188</v>
       </c>
       <c r="F18" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46219</v>
       </c>
       <c r="I18">
@@ -1845,13 +1819,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>90</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1886,13 +1860,13 @@
       <c r="D20">
         <v>56</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46259</v>
       </c>
       <c r="F20" t="s">
         <v>91</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46292</v>
       </c>
       <c r="I20">
@@ -1924,13 +1898,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1965,13 +1939,13 @@
       <c r="D22">
         <v>71</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>46310</v>
       </c>
       <c r="F22" t="s">
         <v>93</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>46342</v>
       </c>
       <c r="I22">
@@ -2003,13 +1977,13 @@
       <c r="D23">
         <v>402</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45791</v>
       </c>
       <c r="F23" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45834</v>
       </c>
       <c r="I23">
@@ -2044,13 +2018,13 @@
       <c r="D24">
         <v>447</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45814</v>
       </c>
       <c r="F24" t="s">
         <v>95</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45955</v>
       </c>
       <c r="I24">
@@ -2088,13 +2062,13 @@
       <c r="D25">
         <v>529</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45853</v>
       </c>
       <c r="F25" t="s">
         <v>85</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45939</v>
       </c>
       <c r="I25">
@@ -2132,13 +2106,13 @@
       <c r="D26">
         <v>691</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45910</v>
       </c>
       <c r="F26" t="s">
         <v>85</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45941</v>
       </c>
       <c r="I26">
@@ -2176,13 +2150,13 @@
       <c r="D27">
         <v>677</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45904</v>
       </c>
       <c r="F27" t="s">
         <v>76</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2217,13 +2191,13 @@
       <c r="D28">
         <v>1278</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46008</v>
       </c>
       <c r="F28" t="s">
         <v>96</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46066</v>
       </c>
       <c r="I28">
@@ -2258,13 +2232,13 @@
       <c r="D29">
         <v>748</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45930</v>
       </c>
       <c r="F29" t="s">
         <v>97</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45991</v>
       </c>
       <c r="I29">
@@ -2299,13 +2273,13 @@
       <c r="D30">
         <v>822</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>45968</v>
       </c>
       <c r="F30" t="s">
         <v>98</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46001</v>
       </c>
       <c r="I30">
@@ -2340,13 +2314,13 @@
       <c r="D31">
         <v>1360</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46043</v>
       </c>
       <c r="F31" t="s">
         <v>84</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46075</v>
       </c>
       <c r="I31">
@@ -2378,13 +2352,13 @@
       <c r="D32">
         <v>2243</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>99</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2419,13 +2393,13 @@
       <c r="D33">
         <v>2245</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>99</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2460,13 +2434,13 @@
       <c r="D34">
         <v>2244</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46289</v>
       </c>
       <c r="F34" t="s">
         <v>99</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46325</v>
       </c>
       <c r="I34">
@@ -2521,13 +2495,13 @@
       <c r="D36">
         <v>1465</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46076</v>
       </c>
       <c r="F36" t="s">
         <v>84</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46106</v>
       </c>
       <c r="I36">
@@ -2559,13 +2533,13 @@
       <c r="D37">
         <v>1882</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>46199</v>
       </c>
       <c r="F37" t="s">
         <v>90</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46233</v>
       </c>
       <c r="I37">
@@ -2601,19 +2575,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>140</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>141</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>142</v>
       </c>
     </row>
@@ -3058,7 +3032,7 @@
       <c r="A42" t="s">
         <v>171</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="1">
         <v>45813</v>
       </c>
     </row>
@@ -3066,7 +3040,7 @@
       <c r="A43" t="s">
         <v>172</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="1">
         <v>45813</v>
       </c>
     </row>
@@ -3074,7 +3048,7 @@
       <c r="A44" t="s">
         <v>173</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="1">
         <v>45842</v>
       </c>
     </row>
@@ -3082,7 +3056,7 @@
       <c r="A45" t="s">
         <v>174</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="1">
         <v>45862</v>
       </c>
     </row>
@@ -3090,7 +3064,7 @@
       <c r="A46" t="s">
         <v>175</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="1">
         <v>45993</v>
       </c>
     </row>
@@ -3122,7 +3096,7 @@
       <c r="A50" t="s">
         <v>179</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -3146,7 +3120,7 @@
       <c r="A53" t="s">
         <v>182</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="1">
         <v>45889</v>
       </c>
     </row>
@@ -3154,7 +3128,7 @@
       <c r="A54" t="s">
         <v>183</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="1">
         <v>45931</v>
       </c>
     </row>
@@ -3194,7 +3168,7 @@
       <c r="A59" t="s">
         <v>188</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="1">
         <v>45980</v>
       </c>
     </row>
@@ -3202,7 +3176,7 @@
       <c r="A60" t="s">
         <v>189</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="1">
         <v>45930</v>
       </c>
     </row>
@@ -3210,7 +3184,7 @@
       <c r="A61" t="s">
         <v>190</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="1">
         <v>45993</v>
       </c>
     </row>
@@ -3234,7 +3208,7 @@
       <c r="A64" t="s">
         <v>193</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="1">
         <v>45993</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (23/10/2026 14:21)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -647,8 +647,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -664,7 +672,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -672,12 +680,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -977,37 +1003,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1057,58 +1083,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1125,13 +1151,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1166,13 +1192,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1207,13 +1233,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1248,13 +1274,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1289,13 +1315,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1333,13 +1359,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1374,13 +1400,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>79</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45955</v>
       </c>
       <c r="I8">
@@ -1415,13 +1441,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>80</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1453,13 +1479,13 @@
       <c r="D10">
         <v>715</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1494,13 +1520,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1535,13 +1561,13 @@
       <c r="D12">
         <v>5</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>83</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46073</v>
       </c>
       <c r="I12">
@@ -1576,13 +1602,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1614,13 +1640,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1655,13 +1681,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>86</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1696,13 +1722,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1737,13 +1763,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>88</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1778,13 +1804,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46188</v>
       </c>
       <c r="F18" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46219</v>
       </c>
       <c r="I18">
@@ -1819,13 +1845,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>90</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1860,13 +1886,13 @@
       <c r="D20">
         <v>56</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46259</v>
       </c>
       <c r="F20" t="s">
         <v>91</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46292</v>
       </c>
       <c r="I20">
@@ -1898,13 +1924,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1939,13 +1965,13 @@
       <c r="D22">
         <v>71</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>46310</v>
       </c>
       <c r="F22" t="s">
         <v>93</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>46342</v>
       </c>
       <c r="I22">
@@ -1977,13 +2003,13 @@
       <c r="D23">
         <v>402</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45791</v>
       </c>
       <c r="F23" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45834</v>
       </c>
       <c r="I23">
@@ -2018,13 +2044,13 @@
       <c r="D24">
         <v>447</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45814</v>
       </c>
       <c r="F24" t="s">
         <v>95</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45955</v>
       </c>
       <c r="I24">
@@ -2062,13 +2088,13 @@
       <c r="D25">
         <v>529</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45853</v>
       </c>
       <c r="F25" t="s">
         <v>85</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45939</v>
       </c>
       <c r="I25">
@@ -2106,13 +2132,13 @@
       <c r="D26">
         <v>691</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45910</v>
       </c>
       <c r="F26" t="s">
         <v>85</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45941</v>
       </c>
       <c r="I26">
@@ -2150,13 +2176,13 @@
       <c r="D27">
         <v>677</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45904</v>
       </c>
       <c r="F27" t="s">
         <v>76</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2191,13 +2217,13 @@
       <c r="D28">
         <v>1278</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46008</v>
       </c>
       <c r="F28" t="s">
         <v>96</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46066</v>
       </c>
       <c r="I28">
@@ -2232,13 +2258,13 @@
       <c r="D29">
         <v>748</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>45930</v>
       </c>
       <c r="F29" t="s">
         <v>97</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>45991</v>
       </c>
       <c r="I29">
@@ -2273,13 +2299,13 @@
       <c r="D30">
         <v>822</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="2">
         <v>45968</v>
       </c>
       <c r="F30" t="s">
         <v>98</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="2">
         <v>46001</v>
       </c>
       <c r="I30">
@@ -2314,13 +2340,13 @@
       <c r="D31">
         <v>1360</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46043</v>
       </c>
       <c r="F31" t="s">
         <v>84</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46075</v>
       </c>
       <c r="I31">
@@ -2352,13 +2378,13 @@
       <c r="D32">
         <v>2243</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>99</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2393,13 +2419,13 @@
       <c r="D33">
         <v>2245</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>99</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2434,13 +2460,13 @@
       <c r="D34">
         <v>2244</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46289</v>
       </c>
       <c r="F34" t="s">
         <v>99</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46325</v>
       </c>
       <c r="I34">
@@ -2495,13 +2521,13 @@
       <c r="D36">
         <v>1465</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="2">
         <v>46076</v>
       </c>
       <c r="F36" t="s">
         <v>84</v>
       </c>
-      <c r="H36" s="1">
+      <c r="H36" s="2">
         <v>46106</v>
       </c>
       <c r="I36">
@@ -2533,13 +2559,13 @@
       <c r="D37">
         <v>1882</v>
       </c>
-      <c r="E37" s="1">
+      <c r="E37" s="2">
         <v>46199</v>
       </c>
       <c r="F37" t="s">
         <v>90</v>
       </c>
-      <c r="H37" s="1">
+      <c r="H37" s="2">
         <v>46233</v>
       </c>
       <c r="I37">
@@ -2575,19 +2601,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>142</v>
       </c>
     </row>
@@ -3032,7 +3058,7 @@
       <c r="A42" t="s">
         <v>171</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="2">
         <v>45813</v>
       </c>
     </row>
@@ -3040,7 +3066,7 @@
       <c r="A43" t="s">
         <v>172</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="2">
         <v>45813</v>
       </c>
     </row>
@@ -3048,7 +3074,7 @@
       <c r="A44" t="s">
         <v>173</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="2">
         <v>45842</v>
       </c>
     </row>
@@ -3056,7 +3082,7 @@
       <c r="A45" t="s">
         <v>174</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="2">
         <v>45862</v>
       </c>
     </row>
@@ -3064,7 +3090,7 @@
       <c r="A46" t="s">
         <v>175</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="2">
         <v>45993</v>
       </c>
     </row>
@@ -3096,7 +3122,7 @@
       <c r="A50" t="s">
         <v>179</v>
       </c>
-      <c r="B50" s="1">
+      <c r="B50" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -3120,7 +3146,7 @@
       <c r="A53" t="s">
         <v>182</v>
       </c>
-      <c r="B53" s="1">
+      <c r="B53" s="2">
         <v>45889</v>
       </c>
     </row>
@@ -3128,7 +3154,7 @@
       <c r="A54" t="s">
         <v>183</v>
       </c>
-      <c r="B54" s="1">
+      <c r="B54" s="2">
         <v>45931</v>
       </c>
     </row>
@@ -3168,7 +3194,7 @@
       <c r="A59" t="s">
         <v>188</v>
       </c>
-      <c r="B59" s="1">
+      <c r="B59" s="2">
         <v>45980</v>
       </c>
     </row>
@@ -3176,7 +3202,7 @@
       <c r="A60" t="s">
         <v>189</v>
       </c>
-      <c r="B60" s="1">
+      <c r="B60" s="2">
         <v>45930</v>
       </c>
     </row>
@@ -3184,7 +3210,7 @@
       <c r="A61" t="s">
         <v>190</v>
       </c>
-      <c r="B61" s="1">
+      <c r="B61" s="2">
         <v>45993</v>
       </c>
     </row>
@@ -3208,7 +3234,7 @@
       <c r="A64" t="s">
         <v>193</v>
       </c>
-      <c r="B64" s="1">
+      <c r="B64" s="2">
         <v>45993</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (26/10/2026 14:17)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -647,16 +647,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -672,7 +664,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -680,30 +672,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1003,37 +977,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1083,58 +1057,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1151,13 +1125,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1192,13 +1166,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1233,13 +1207,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1274,13 +1248,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1315,13 +1289,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1359,13 +1333,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1400,13 +1374,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>79</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45955</v>
       </c>
       <c r="I8">
@@ -1441,13 +1415,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>80</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1479,13 +1453,13 @@
       <c r="D10">
         <v>715</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1520,13 +1494,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1561,13 +1535,13 @@
       <c r="D12">
         <v>5</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>83</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46073</v>
       </c>
       <c r="I12">
@@ -1602,13 +1576,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1640,13 +1614,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1681,13 +1655,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>86</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1722,13 +1696,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1763,13 +1737,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>88</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1804,13 +1778,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46188</v>
       </c>
       <c r="F18" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46219</v>
       </c>
       <c r="I18">
@@ -1845,13 +1819,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>90</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1886,13 +1860,13 @@
       <c r="D20">
         <v>56</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46259</v>
       </c>
       <c r="F20" t="s">
         <v>91</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46292</v>
       </c>
       <c r="I20">
@@ -1924,13 +1898,13 @@
       <c r="D21">
         <v>66</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>46280</v>
       </c>
       <c r="F21" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>46312</v>
       </c>
       <c r="I21">
@@ -1965,13 +1939,13 @@
       <c r="D22">
         <v>71</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>46310</v>
       </c>
       <c r="F22" t="s">
         <v>93</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>46342</v>
       </c>
       <c r="I22">
@@ -2003,13 +1977,13 @@
       <c r="D23">
         <v>402</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45791</v>
       </c>
       <c r="F23" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45834</v>
       </c>
       <c r="I23">
@@ -2044,13 +2018,13 @@
       <c r="D24">
         <v>447</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45814</v>
       </c>
       <c r="F24" t="s">
         <v>95</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45955</v>
       </c>
       <c r="I24">
@@ -2088,13 +2062,13 @@
       <c r="D25">
         <v>529</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45853</v>
       </c>
       <c r="F25" t="s">
         <v>85</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45939</v>
       </c>
       <c r="I25">
@@ -2132,13 +2106,13 @@
       <c r="D26">
         <v>691</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45910</v>
       </c>
       <c r="F26" t="s">
         <v>85</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45941</v>
       </c>
       <c r="I26">
@@ -2176,13 +2150,13 @@
       <c r="D27">
         <v>677</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45904</v>
       </c>
       <c r="F27" t="s">
         <v>76</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2217,13 +2191,13 @@
       <c r="D28">
         <v>1278</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46008</v>
       </c>
       <c r="F28" t="s">
         <v>96</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46066</v>
       </c>
       <c r="I28">
@@ -2258,13 +2232,13 @@
       <c r="D29">
         <v>748</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>45930</v>
       </c>
       <c r="F29" t="s">
         <v>97</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>45991</v>
       </c>
       <c r="I29">
@@ -2299,13 +2273,13 @@
       <c r="D30">
         <v>822</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="1">
         <v>45968</v>
       </c>
       <c r="F30" t="s">
         <v>98</v>
       </c>
-      <c r="H30" s="2">
+      <c r="H30" s="1">
         <v>46001</v>
       </c>
       <c r="I30">
@@ -2340,13 +2314,13 @@
       <c r="D31">
         <v>1360</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46043</v>
       </c>
       <c r="F31" t="s">
         <v>84</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46075</v>
       </c>
       <c r="I31">
@@ -2378,13 +2352,13 @@
       <c r="D32">
         <v>2243</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46289</v>
       </c>
       <c r="F32" t="s">
         <v>99</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46325</v>
       </c>
       <c r="I32">
@@ -2419,13 +2393,13 @@
       <c r="D33">
         <v>2245</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46289</v>
       </c>
       <c r="F33" t="s">
         <v>99</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46325</v>
       </c>
       <c r="I33">
@@ -2460,13 +2434,13 @@
       <c r="D34">
         <v>2244</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46289</v>
       </c>
       <c r="F34" t="s">
         <v>99</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46325</v>
       </c>
       <c r="I34">
@@ -2521,13 +2495,13 @@
       <c r="D36">
         <v>1465</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36" s="1">
         <v>46076</v>
       </c>
       <c r="F36" t="s">
         <v>84</v>
       </c>
-      <c r="H36" s="2">
+      <c r="H36" s="1">
         <v>46106</v>
       </c>
       <c r="I36">
@@ -2559,13 +2533,13 @@
       <c r="D37">
         <v>1882</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37" s="1">
         <v>46199</v>
       </c>
       <c r="F37" t="s">
         <v>90</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="1">
         <v>46233</v>
       </c>
       <c r="I37">
@@ -2601,19 +2575,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>140</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>141</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>142</v>
       </c>
     </row>
@@ -3058,7 +3032,7 @@
       <c r="A42" t="s">
         <v>171</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="1">
         <v>45813</v>
       </c>
     </row>
@@ -3066,7 +3040,7 @@
       <c r="A43" t="s">
         <v>172</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="1">
         <v>45813</v>
       </c>
     </row>
@@ -3074,7 +3048,7 @@
       <c r="A44" t="s">
         <v>173</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="1">
         <v>45842</v>
       </c>
     </row>
@@ -3082,7 +3056,7 @@
       <c r="A45" t="s">
         <v>174</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="1">
         <v>45862</v>
       </c>
     </row>
@@ -3090,7 +3064,7 @@
       <c r="A46" t="s">
         <v>175</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="1">
         <v>45993</v>
       </c>
     </row>
@@ -3122,7 +3096,7 @@
       <c r="A50" t="s">
         <v>179</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -3146,7 +3120,7 @@
       <c r="A53" t="s">
         <v>182</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="1">
         <v>45889</v>
       </c>
     </row>
@@ -3154,7 +3128,7 @@
       <c r="A54" t="s">
         <v>183</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="1">
         <v>45931</v>
       </c>
     </row>
@@ -3194,7 +3168,7 @@
       <c r="A59" t="s">
         <v>188</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="1">
         <v>45980</v>
       </c>
     </row>
@@ -3202,7 +3176,7 @@
       <c r="A60" t="s">
         <v>189</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="1">
         <v>45930</v>
       </c>
     </row>
@@ -3210,7 +3184,7 @@
       <c r="A61" t="s">
         <v>190</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="1">
         <v>45993</v>
       </c>
     </row>
@@ -3234,7 +3208,7 @@
       <c r="A64" t="s">
         <v>193</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="1">
         <v>45993</v>
       </c>
     </row>

</xml_diff>